<commit_message>
Yayın: proje adı bütün evrakta tek kaynağa bağlandı
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
+++ b/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="F13" s="20" t="n">
-        <v>38.71</v>
+        <v>44.0481</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>72192.55</v>
@@ -1843,7 +1843,7 @@
         <v>1</v>
       </c>
       <c r="G33" s="5" t="n">
-        <v>9209.41</v>
+        <v>10082.96</v>
       </c>
       <c r="H33" s="5">
         <f>F33*G33</f>
@@ -1880,7 +1880,7 @@
         <v>1</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>4586.47</v>
+        <v>4435.25</v>
       </c>
       <c r="H34" s="5">
         <f>F34*G34</f>
@@ -1917,7 +1917,7 @@
         <v>2</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>1402.96</v>
+        <v>1436.2</v>
       </c>
       <c r="H35" s="5">
         <f>F35*G35</f>
@@ -1954,7 +1954,7 @@
         <v>300</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>260.01</v>
+        <v>244.02</v>
       </c>
       <c r="H36" s="5">
         <f>F36*G36</f>
@@ -1991,7 +1991,7 @@
         <v>30</v>
       </c>
       <c r="G37" s="5" t="n">
-        <v>2594.89</v>
+        <v>2222.88</v>
       </c>
       <c r="H37" s="5">
         <f>F37*G37</f>
@@ -2028,7 +2028,7 @@
         <v>2</v>
       </c>
       <c r="G38" s="5" t="n">
-        <v>1782.25</v>
+        <v>1552.4</v>
       </c>
       <c r="H38" s="5">
         <f>F38*G38</f>
@@ -2065,7 +2065,7 @@
         <v>500</v>
       </c>
       <c r="G39" s="5" t="n">
-        <v>37.77</v>
+        <v>74.42</v>
       </c>
       <c r="H39" s="5">
         <f>F39*G39</f>
@@ -2102,7 +2102,7 @@
         <v>2000</v>
       </c>
       <c r="G40" s="5" t="n">
-        <v>25.35</v>
+        <v>33.1</v>
       </c>
       <c r="H40" s="5">
         <f>F40*G40</f>
@@ -2139,7 +2139,7 @@
         <v>600</v>
       </c>
       <c r="G41" s="5" t="n">
-        <v>15.88</v>
+        <v>23.56</v>
       </c>
       <c r="H41" s="5">
         <f>F41*G41</f>
@@ -2176,7 +2176,7 @@
         <v>100</v>
       </c>
       <c r="G42" s="5" t="n">
-        <v>204.16</v>
+        <v>188.13</v>
       </c>
       <c r="H42" s="5">
         <f>F42*G42</f>
@@ -2213,7 +2213,7 @@
         <v>186</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>150.75</v>
+        <v>156.11</v>
       </c>
       <c r="H43" s="5">
         <f>F43*G43</f>
@@ -2250,7 +2250,7 @@
         <v>1</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>20274.29</v>
+        <v>17410.01</v>
       </c>
       <c r="H44" s="5">
         <f>F44*G44</f>
@@ -2287,7 +2287,7 @@
         <v>16</v>
       </c>
       <c r="G45" s="5" t="n">
-        <v>554.74</v>
+        <v>481.15</v>
       </c>
       <c r="H45" s="5">
         <f>F45*G45</f>
@@ -2324,7 +2324,7 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>607554.0699999999</v>
+        <v>484082.09</v>
       </c>
       <c r="H46" s="5">
         <f>F46*G46</f>
@@ -2361,7 +2361,7 @@
         <v>1</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>103549.61</v>
+        <v>83282.35000000001</v>
       </c>
       <c r="H47" s="5">
         <f>F47*G47</f>
@@ -2398,7 +2398,7 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>50107.49</v>
+        <v>44709.81</v>
       </c>
       <c r="H48" s="5">
         <f>F48*G48</f>
@@ -2728,7 +2728,7 @@
         </is>
       </c>
       <c r="F57" s="20" t="n">
-        <v>38.71</v>
+        <v>44.0481</v>
       </c>
       <c r="G57" s="5" t="n">
         <v>72192.55</v>
@@ -3471,7 +3471,7 @@
         <v>1</v>
       </c>
       <c r="G77" s="5" t="n">
-        <v>9209.41</v>
+        <v>10082.96</v>
       </c>
       <c r="H77" s="5">
         <f>F77*G77</f>
@@ -3508,7 +3508,7 @@
         <v>1</v>
       </c>
       <c r="G78" s="5" t="n">
-        <v>4586.47</v>
+        <v>4435.25</v>
       </c>
       <c r="H78" s="5">
         <f>F78*G78</f>
@@ -3545,7 +3545,7 @@
         <v>2</v>
       </c>
       <c r="G79" s="5" t="n">
-        <v>1402.96</v>
+        <v>1436.2</v>
       </c>
       <c r="H79" s="5">
         <f>F79*G79</f>
@@ -3582,7 +3582,7 @@
         <v>300</v>
       </c>
       <c r="G80" s="5" t="n">
-        <v>260.01</v>
+        <v>244.02</v>
       </c>
       <c r="H80" s="5">
         <f>F80*G80</f>
@@ -3619,7 +3619,7 @@
         <v>30</v>
       </c>
       <c r="G81" s="5" t="n">
-        <v>2594.89</v>
+        <v>2222.88</v>
       </c>
       <c r="H81" s="5">
         <f>F81*G81</f>
@@ -3656,7 +3656,7 @@
         <v>2</v>
       </c>
       <c r="G82" s="5" t="n">
-        <v>1782.25</v>
+        <v>1552.4</v>
       </c>
       <c r="H82" s="5">
         <f>F82*G82</f>
@@ -3693,7 +3693,7 @@
         <v>500</v>
       </c>
       <c r="G83" s="5" t="n">
-        <v>37.77</v>
+        <v>74.42</v>
       </c>
       <c r="H83" s="5">
         <f>F83*G83</f>
@@ -3730,7 +3730,7 @@
         <v>2000</v>
       </c>
       <c r="G84" s="5" t="n">
-        <v>25.35</v>
+        <v>33.1</v>
       </c>
       <c r="H84" s="5">
         <f>F84*G84</f>
@@ -3767,7 +3767,7 @@
         <v>600</v>
       </c>
       <c r="G85" s="5" t="n">
-        <v>15.88</v>
+        <v>23.56</v>
       </c>
       <c r="H85" s="5">
         <f>F85*G85</f>
@@ -3804,7 +3804,7 @@
         <v>100</v>
       </c>
       <c r="G86" s="5" t="n">
-        <v>204.16</v>
+        <v>188.13</v>
       </c>
       <c r="H86" s="5">
         <f>F86*G86</f>
@@ -3841,7 +3841,7 @@
         <v>186</v>
       </c>
       <c r="G87" s="5" t="n">
-        <v>150.75</v>
+        <v>156.11</v>
       </c>
       <c r="H87" s="5">
         <f>F87*G87</f>
@@ -3878,7 +3878,7 @@
         <v>1</v>
       </c>
       <c r="G88" s="5" t="n">
-        <v>20274.29</v>
+        <v>17410.01</v>
       </c>
       <c r="H88" s="5">
         <f>F88*G88</f>
@@ -3915,7 +3915,7 @@
         <v>16</v>
       </c>
       <c r="G89" s="5" t="n">
-        <v>554.74</v>
+        <v>481.15</v>
       </c>
       <c r="H89" s="5">
         <f>F89*G89</f>
@@ -3952,7 +3952,7 @@
         <v>1</v>
       </c>
       <c r="G90" s="5" t="n">
-        <v>607554.0699999999</v>
+        <v>484082.09</v>
       </c>
       <c r="H90" s="5">
         <f>F90*G90</f>
@@ -3989,7 +3989,7 @@
         <v>1</v>
       </c>
       <c r="G91" s="5" t="n">
-        <v>103549.61</v>
+        <v>83282.35000000001</v>
       </c>
       <c r="H91" s="5">
         <f>F91*G91</f>
@@ -4026,7 +4026,7 @@
         <v>1</v>
       </c>
       <c r="G92" s="5" t="n">
-        <v>50107.49</v>
+        <v>44709.81</v>
       </c>
       <c r="H92" s="5">
         <f>F92*G92</f>
@@ -5321,7 +5321,7 @@
         <v>1</v>
       </c>
       <c r="G127" s="5" t="n">
-        <v>41083.03</v>
+        <v>41783.13</v>
       </c>
       <c r="H127" s="5">
         <f>F127*G127</f>
@@ -5358,7 +5358,7 @@
         <v>1</v>
       </c>
       <c r="G128" s="5" t="n">
-        <v>10633.02</v>
+        <v>11631.65</v>
       </c>
       <c r="H128" s="5">
         <f>F128*G128</f>
@@ -5395,7 +5395,7 @@
         <v>1</v>
       </c>
       <c r="G129" s="5" t="n">
-        <v>1955.4</v>
+        <v>2218.15</v>
       </c>
       <c r="H129" s="5">
         <f>F129*G129</f>
@@ -5432,7 +5432,7 @@
         <v>1</v>
       </c>
       <c r="G130" s="5" t="n">
-        <v>6179.11</v>
+        <v>5920.76</v>
       </c>
       <c r="H130" s="5">
         <f>F130*G130</f>
@@ -5469,7 +5469,7 @@
         <v>2</v>
       </c>
       <c r="G131" s="5" t="n">
-        <v>1402.96</v>
+        <v>1436.2</v>
       </c>
       <c r="H131" s="5">
         <f>F131*G131</f>
@@ -5506,7 +5506,7 @@
         <v>50</v>
       </c>
       <c r="G132" s="5" t="n">
-        <v>360.29</v>
+        <v>332.17</v>
       </c>
       <c r="H132" s="5">
         <f>F132*G132</f>
@@ -5543,7 +5543,7 @@
         <v>50</v>
       </c>
       <c r="G133" s="5" t="n">
-        <v>66.63</v>
+        <v>71.31999999999999</v>
       </c>
       <c r="H133" s="5">
         <f>F133*G133</f>
@@ -5580,7 +5580,7 @@
         <v>4</v>
       </c>
       <c r="G134" s="5" t="n">
-        <v>8097.86</v>
+        <v>7783.12</v>
       </c>
       <c r="H134" s="5">
         <f>F134*G134</f>
@@ -5617,7 +5617,7 @@
         <v>4</v>
       </c>
       <c r="G135" s="5" t="n">
-        <v>9922.59</v>
+        <v>8313.16</v>
       </c>
       <c r="H135" s="5">
         <f>F135*G135</f>
@@ -6584,7 +6584,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>23916998.24</v>
+        <v>24418682.03</v>
       </c>
       <c r="C5" s="6">
         <f>B5/52.7585</f>
@@ -6622,7 +6622,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>4132560.74</v>
+        <v>4634244.53</v>
       </c>
       <c r="C7" s="14">
         <f>B7/52.7585</f>
@@ -6641,7 +6641,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>4783399.65</v>
+        <v>4883736.41</v>
       </c>
       <c r="C8" s="6">
         <f>B8/52.7585</f>

</xml_diff>

<commit_message>
Yayın: ekipman adetleri mekanik projeye indirildi
Tünel fanı 7 -> 4 adet/kümes, panjur klapesi 80 -> 40 adet/kümes.
Makine-ekipman tutarı 3.344.220,00 -> 3.095.220,00 TL.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
+++ b/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
@@ -6584,7 +6584,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>24418682.03</v>
+        <v>24169682.03</v>
       </c>
       <c r="C5" s="6">
         <f>B5/52.7585</f>
@@ -6622,7 +6622,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>4634244.53</v>
+        <v>4385244.53</v>
       </c>
       <c r="C7" s="14">
         <f>B7/52.7585</f>
@@ -6641,7 +6641,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>4883736.41</v>
+        <v>4833936.41</v>
       </c>
       <c r="C8" s="6">
         <f>B8/52.7585</f>

</xml_diff>

<commit_message>
Yayın: proforma belgeleri eklendi (48 belge)
Proforma listesi ve üç proforma fatura; ısıtma sistemi uygun olmayan
harcamaya dahil edildi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
+++ b/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -736,40 +736,59 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Hibe dışı kümes ısıtma sistemi</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>710000</v>
+      </c>
+      <c r="C14" s="6">
+        <f>B14/52.7585</f>
+        <v/>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Ayrı lot; proforma ile beyan</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>UYGUN OLMAYAN HARCAMA (öz kaynak)</t>
         </is>
       </c>
-      <c r="B14" s="9">
-        <f>B12+B13</f>
-        <v/>
-      </c>
-      <c r="C14" s="10">
-        <f>B14/52.7585</f>
-        <v/>
-      </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="B15" s="9">
+        <f>B12+B13+B14</f>
+        <v/>
+      </c>
+      <c r="C15" s="10">
+        <f>B15/52.7585</f>
+        <v/>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>Tamamı öz kaynaktan karşılanır</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>TOPLAM YATIRIM (KDV hariç)</t>
         </is>
       </c>
-      <c r="B15" s="13">
-        <f>B9+B14</f>
-        <v/>
-      </c>
-      <c r="C15" s="14">
-        <f>B15/52.7585</f>
-        <v/>
-      </c>
-      <c r="D15" s="15" t="inlineStr">
+      <c r="B16" s="13">
+        <f>B9+B15</f>
+        <v/>
+      </c>
+      <c r="C16" s="14">
+        <f>B16/52.7585</f>
+        <v/>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
         <is>
           <t>Uygun harcama + uygun olmayan harcama</t>
         </is>
@@ -6843,7 +6862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="66" customWidth="1" min="1" max="1"/>
@@ -6896,7 +6915,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>24169695.26</v>
+        <v>24879695.26</v>
       </c>
       <c r="C5" s="6">
         <f>B5/52.7585</f>
@@ -6966,57 +6985,76 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="24" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>Hibe dışı kümes ısıtma sistemi — ayrı lot</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>710000</v>
+      </c>
+      <c r="C9" s="6">
+        <f>B9/52.7585</f>
+        <v/>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>Proforma fatura</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>UYGUN OLMAYAN HARCAMA — toplam</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n">
-        <v>8592975.42</v>
-      </c>
-      <c r="C9" s="10">
-        <f>B9/52.7585</f>
-        <v/>
-      </c>
-      <c r="D9" s="25" t="inlineStr">
+      <c r="B10" s="9" t="n">
+        <v>9302975.42</v>
+      </c>
+      <c r="C10" s="10">
+        <f>B10/52.7585</f>
+        <v/>
+      </c>
+      <c r="D10" s="25" t="inlineStr">
         <is>
           <t>Öz kaynak</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>IPARD III broyler uygun harcama üst limiti (375.000,00 Avro) — uygun harcama limitin altındadır</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>19784437.5</v>
-      </c>
-      <c r="C10" s="6">
-        <f>B10/52.7585</f>
-        <v/>
-      </c>
-      <c r="D10" s="17" t="inlineStr">
-        <is>
-          <t>Çağrı rehberi</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>KDV — IPARD'da uygun harcama değildir</t>
+          <t>IPARD III broyler uygun harcama üst limiti (375.000,00 Avro) — uygun harcama limitin altındadır</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>4833939.05</v>
+        <v>19784437.5</v>
       </c>
       <c r="C11" s="6">
         <f>B11/52.7585</f>
         <v/>
       </c>
       <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>Çağrı rehberi</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>KDV — IPARD'da uygun harcama değildir</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>4975939.05</v>
+      </c>
+      <c r="C12" s="6">
+        <f>B12/52.7585</f>
+        <v/>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
         <is>
           <t>Öz kaynak</t>
         </is>

</xml_diff>

<commit_message>
Yayın: yağmur suyu deposu ve proje miktarlı ekipman
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
+++ b/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>'A3.4-EK Yapım'!H51</f>
+        <f>'A3.4-EK Yapım'!H56</f>
         <v/>
       </c>
       <c r="C12" s="6">
@@ -4507,7 +4507,7 @@
         </is>
       </c>
       <c r="E13" s="20" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>1200</v>
@@ -4597,7 +4597,7 @@
         </is>
       </c>
       <c r="E16" s="20" t="n">
-        <v>90</v>
+        <v>45.72</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>4500</v>
@@ -4757,7 +4757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -5049,25 +5049,25 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="20" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>Beton işleri</t>
+          <t>Kazı, dolgu ve reglaj işleri</t>
         </is>
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>Gübre Çukuru</t>
+          <t>Yağmur Suyu Deposu</t>
         </is>
       </c>
       <c r="C11" s="18" t="inlineStr">
         <is>
-          <t>15.150.1003</t>
+          <t>15.120.1101</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>Beton santralinde üretilen veya satın alınan ve beton pompasıyla basılan, C 16/20 basınç dayanım sınıfında, gri renkte, normal hazır beton dökülmesi (beton nakli dahil)</t>
+          <t>Makine ile her derinlik ve her genişlikte yumuşak ve sert toprak kazılması</t>
         </is>
       </c>
       <c r="E11" s="19" t="inlineStr">
@@ -5076,10 +5076,10 @@
         </is>
       </c>
       <c r="F11" s="20" t="n">
-        <v>11.934</v>
+        <v>88.75</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>2750.454</v>
+        <v>60.354</v>
       </c>
       <c r="H11" s="5">
         <f>F11*G11</f>
@@ -5094,7 +5094,7 @@
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>Ölü Atma Çukuru</t>
+          <t>Gübre Çukuru</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
@@ -5113,7 +5113,7 @@
         </is>
       </c>
       <c r="F12" s="20" t="n">
-        <v>1.984</v>
+        <v>11.934</v>
       </c>
       <c r="G12" s="5" t="n">
         <v>2750.454</v>
@@ -5131,7 +5131,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>Foseptik</t>
+          <t>Ölü Atma Çukuru</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -5150,7 +5150,7 @@
         </is>
       </c>
       <c r="F13" s="20" t="n">
-        <v>0.484</v>
+        <v>1.984</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>2750.454</v>
@@ -5168,7 +5168,7 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>Yem Silosu Betonarme Kaideleri</t>
+          <t>Foseptik</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
@@ -5187,7 +5187,7 @@
         </is>
       </c>
       <c r="F14" s="20" t="n">
-        <v>1.922</v>
+        <v>0.484</v>
       </c>
       <c r="G14" s="5" t="n">
         <v>2750.454</v>
@@ -5205,7 +5205,7 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>Su Deposu</t>
+          <t>Yem Silosu Betonarme Kaideleri</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
@@ -5224,7 +5224,7 @@
         </is>
       </c>
       <c r="F15" s="20" t="n">
-        <v>1.344</v>
+        <v>1.922</v>
       </c>
       <c r="G15" s="5" t="n">
         <v>2750.454</v>
@@ -5237,22 +5237,22 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>Betonarme işleri</t>
+          <t>Beton işleri</t>
         </is>
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>Gübre Çukuru</t>
+          <t>Su Deposu</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>15.150.1005</t>
+          <t>15.150.1003</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>Beton santralinde üretilen veya satın alınan ve beton pompasıyla basılan, C 25/30 basınç dayanım sınıfında, gri renkte, normal hazır beton dökülmesi (beton nakli dahil)</t>
+          <t>Beton santralinde üretilen veya satın alınan ve beton pompasıyla basılan, C 16/20 basınç dayanım sınıfında, gri renkte, normal hazır beton dökülmesi (beton nakli dahil)</t>
         </is>
       </c>
       <c r="E16" s="19" t="inlineStr">
@@ -5261,10 +5261,10 @@
         </is>
       </c>
       <c r="F16" s="20" t="n">
-        <v>93.19</v>
+        <v>1.344</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>2960.454</v>
+        <v>2750.454</v>
       </c>
       <c r="H16" s="5">
         <f>F16*G16</f>
@@ -5274,22 +5274,22 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>Betonarme işleri</t>
+          <t>Beton işleri</t>
         </is>
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>Ölü Atma Çukuru</t>
+          <t>Yağmur Suyu Deposu</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>15.150.1005</t>
+          <t>15.150.1003</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>Beton santralinde üretilen veya satın alınan ve beton pompasıyla basılan, C 25/30 basınç dayanım sınıfında, gri renkte, normal hazır beton dökülmesi (beton nakli dahil)</t>
+          <t>Beton santralinde üretilen veya satın alınan ve beton pompasıyla basılan, C 16/20 basınç dayanım sınıfında, gri renkte, normal hazır beton dökülmesi (beton nakli dahil)</t>
         </is>
       </c>
       <c r="E17" s="19" t="inlineStr">
@@ -5298,10 +5298,10 @@
         </is>
       </c>
       <c r="F17" s="20" t="n">
-        <v>20.85</v>
+        <v>1.024</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>2960.454</v>
+        <v>2750.454</v>
       </c>
       <c r="H17" s="5">
         <f>F17*G17</f>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>Su Deposu</t>
+          <t>Gübre Çukuru</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
@@ -5335,7 +5335,7 @@
         </is>
       </c>
       <c r="F18" s="20" t="n">
-        <v>15.15</v>
+        <v>93.19</v>
       </c>
       <c r="G18" s="5" t="n">
         <v>2960.454</v>
@@ -5353,7 +5353,7 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>Foseptik</t>
+          <t>Ölü Atma Çukuru</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
@@ -5372,7 +5372,7 @@
         </is>
       </c>
       <c r="F19" s="20" t="n">
-        <v>6.175</v>
+        <v>20.85</v>
       </c>
       <c r="G19" s="5" t="n">
         <v>2960.454</v>
@@ -5390,7 +5390,7 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Yem Silosu Betonarme Kaideleri</t>
+          <t>Su Deposu</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
@@ -5409,7 +5409,7 @@
         </is>
       </c>
       <c r="F20" s="20" t="n">
-        <v>8.41</v>
+        <v>15.15</v>
       </c>
       <c r="G20" s="5" t="n">
         <v>2960.454</v>
@@ -5419,111 +5419,111 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="14" customHeight="1">
+    <row r="21" ht="30" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>Kalıp, yapı iskelesi işleri</t>
+          <t>Betonarme işleri</t>
         </is>
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>Gübre Çukuru</t>
+          <t>Yağmur Suyu Deposu</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>15.180.1003</t>
+          <t>15.150.1005</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr">
         <is>
-          <t>Plywood ile düz yüzeyli betonarme kalıbı yapılması</t>
+          <t>Beton santralinde üretilen veya satın alınan ve beton pompasıyla basılan, C 25/30 basınç dayanım sınıfında, gri renkte, normal hazır beton dökülmesi (beton nakli dahil)</t>
         </is>
       </c>
       <c r="E21" s="19" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="F21" s="20" t="n">
-        <v>363.26</v>
+        <v>12.3</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>863.7972</v>
+        <v>2960.454</v>
       </c>
       <c r="H21" s="5">
         <f>F21*G21</f>
         <v/>
       </c>
     </row>
-    <row r="22" ht="14" customHeight="1">
+    <row r="22" ht="30" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>Kalıp, yapı iskelesi işleri</t>
+          <t>Betonarme işleri</t>
         </is>
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>Ölü Atma Çukuru</t>
+          <t>Foseptik</t>
         </is>
       </c>
       <c r="C22" s="18" t="inlineStr">
         <is>
-          <t>15.180.1003</t>
+          <t>15.150.1005</t>
         </is>
       </c>
       <c r="D22" s="16" t="inlineStr">
         <is>
-          <t>Plywood ile düz yüzeyli betonarme kalıbı yapılması</t>
+          <t>Beton santralinde üretilen veya satın alınan ve beton pompasıyla basılan, C 25/30 basınç dayanım sınıfında, gri renkte, normal hazır beton dökülmesi (beton nakli dahil)</t>
         </is>
       </c>
       <c r="E22" s="19" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="F22" s="20" t="n">
-        <v>127.2</v>
+        <v>6.175</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>863.7972</v>
+        <v>2960.454</v>
       </c>
       <c r="H22" s="5">
         <f>F22*G22</f>
         <v/>
       </c>
     </row>
-    <row r="23" ht="14" customHeight="1">
+    <row r="23" ht="30" customHeight="1">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t>Kalıp, yapı iskelesi işleri</t>
+          <t>Betonarme işleri</t>
         </is>
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>Su Deposu</t>
+          <t>Yem Silosu Betonarme Kaideleri</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>15.180.1003</t>
+          <t>15.150.1005</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
         <is>
-          <t>Plywood ile düz yüzeyli betonarme kalıbı yapılması</t>
+          <t>Beton santralinde üretilen veya satın alınan ve beton pompasıyla basılan, C 25/30 basınç dayanım sınıfında, gri renkte, normal hazır beton dökülmesi (beton nakli dahil)</t>
         </is>
       </c>
       <c r="E23" s="19" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="F23" s="20" t="n">
-        <v>95.59999999999999</v>
+        <v>8.41</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>863.7972</v>
+        <v>2960.454</v>
       </c>
       <c r="H23" s="5">
         <f>F23*G23</f>
@@ -5538,7 +5538,7 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>Foseptik</t>
+          <t>Gübre Çukuru</t>
         </is>
       </c>
       <c r="C24" s="18" t="inlineStr">
@@ -5557,7 +5557,7 @@
         </is>
       </c>
       <c r="F24" s="20" t="n">
-        <v>41.4</v>
+        <v>363.26</v>
       </c>
       <c r="G24" s="5" t="n">
         <v>863.7972</v>
@@ -5575,7 +5575,7 @@
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>Yem Silosu Betonarme Kaideleri</t>
+          <t>Ölü Atma Çukuru</t>
         </is>
       </c>
       <c r="C25" s="18" t="inlineStr">
@@ -5594,7 +5594,7 @@
         </is>
       </c>
       <c r="F25" s="20" t="n">
-        <v>11.6</v>
+        <v>127.2</v>
       </c>
       <c r="G25" s="5" t="n">
         <v>863.7972</v>
@@ -5604,148 +5604,148 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="20" customHeight="1">
+    <row r="26" ht="14" customHeight="1">
       <c r="A26" s="16" t="inlineStr">
         <is>
-          <t>Demir-inşaat işleri</t>
+          <t>Kalıp, yapı iskelesi işleri</t>
         </is>
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>Gübre Çukuru</t>
+          <t>Su Deposu</t>
         </is>
       </c>
       <c r="C26" s="18" t="inlineStr">
         <is>
-          <t>15.160.1003</t>
+          <t>15.180.1003</t>
         </is>
       </c>
       <c r="D26" s="16" t="inlineStr">
         <is>
-          <t>Ø 8 - Ø 12 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
+          <t>Plywood ile düz yüzeyli betonarme kalıbı yapılması</t>
         </is>
       </c>
       <c r="E26" s="19" t="inlineStr">
         <is>
-          <t>ton</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="F26" s="20" t="n">
-        <v>7.599</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>39045.2412</v>
+        <v>863.7972</v>
       </c>
       <c r="H26" s="5">
         <f>F26*G26</f>
         <v/>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
+    <row r="27" ht="14" customHeight="1">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>Demir-inşaat işleri</t>
+          <t>Kalıp, yapı iskelesi işleri</t>
         </is>
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>Gübre Çukuru</t>
+          <t>Yağmur Suyu Deposu</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>15.160.1004</t>
+          <t>15.180.1003</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>Ø 14 - Ø 28 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
+          <t>Plywood ile düz yüzeyli betonarme kalıbı yapılması</t>
         </is>
       </c>
       <c r="E27" s="19" t="inlineStr">
         <is>
-          <t>ton</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="F27" s="20" t="n">
-        <v>0.5639999999999999</v>
+        <v>79.8</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>37532.1912</v>
+        <v>863.7972</v>
       </c>
       <c r="H27" s="5">
         <f>F27*G27</f>
         <v/>
       </c>
     </row>
-    <row r="28" ht="20" customHeight="1">
+    <row r="28" ht="14" customHeight="1">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>Demir-inşaat işleri</t>
+          <t>Kalıp, yapı iskelesi işleri</t>
         </is>
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>Ölü Atma Çukuru</t>
+          <t>Foseptik</t>
         </is>
       </c>
       <c r="C28" s="18" t="inlineStr">
         <is>
-          <t>15.160.1003</t>
+          <t>15.180.1003</t>
         </is>
       </c>
       <c r="D28" s="16" t="inlineStr">
         <is>
-          <t>Ø 8 - Ø 12 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
+          <t>Plywood ile düz yüzeyli betonarme kalıbı yapılması</t>
         </is>
       </c>
       <c r="E28" s="19" t="inlineStr">
         <is>
-          <t>ton</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="F28" s="20" t="n">
-        <v>1.657</v>
+        <v>41.4</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>39045.2412</v>
+        <v>863.7972</v>
       </c>
       <c r="H28" s="5">
         <f>F28*G28</f>
         <v/>
       </c>
     </row>
-    <row r="29" ht="20" customHeight="1">
+    <row r="29" ht="14" customHeight="1">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t>Demir-inşaat işleri</t>
+          <t>Kalıp, yapı iskelesi işleri</t>
         </is>
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>Foseptik</t>
+          <t>Yem Silosu Betonarme Kaideleri</t>
         </is>
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>15.160.1003</t>
+          <t>15.180.1003</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>Ø 8 - Ø 12 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
+          <t>Plywood ile düz yüzeyli betonarme kalıbı yapılması</t>
         </is>
       </c>
       <c r="E29" s="19" t="inlineStr">
         <is>
-          <t>ton</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="F29" s="20" t="n">
-        <v>0.587</v>
+        <v>11.6</v>
       </c>
       <c r="G29" s="5" t="n">
-        <v>39045.2412</v>
+        <v>863.7972</v>
       </c>
       <c r="H29" s="5">
         <f>F29*G29</f>
@@ -5760,7 +5760,7 @@
       </c>
       <c r="B30" s="17" t="inlineStr">
         <is>
-          <t>Yem Silosu Betonarme Kaideleri</t>
+          <t>Gübre Çukuru</t>
         </is>
       </c>
       <c r="C30" s="18" t="inlineStr">
@@ -5779,7 +5779,7 @@
         </is>
       </c>
       <c r="F30" s="20" t="n">
-        <v>0.757</v>
+        <v>7.599</v>
       </c>
       <c r="G30" s="5" t="n">
         <v>39045.2412</v>
@@ -5797,17 +5797,17 @@
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>Su Deposu</t>
+          <t>Gübre Çukuru</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>15.160.1003</t>
+          <t>15.160.1004</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
-          <t>Ø 8 - Ø 12 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
+          <t>Ø 14 - Ø 28 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
         </is>
       </c>
       <c r="E31" s="19" t="inlineStr">
@@ -5816,121 +5816,121 @@
         </is>
       </c>
       <c r="F31" s="20" t="n">
-        <v>1.232</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G31" s="5" t="n">
-        <v>39045.2412</v>
+        <v>37532.1912</v>
       </c>
       <c r="H31" s="5">
         <f>F31*G31</f>
         <v/>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1">
+    <row r="32" ht="20" customHeight="1">
       <c r="A32" s="16" t="inlineStr">
         <is>
-          <t>Çatı ve sundurma işleri</t>
+          <t>Demir-inşaat işleri</t>
         </is>
       </c>
       <c r="B32" s="17" t="inlineStr">
         <is>
-          <t>Kümes A Blok</t>
+          <t>Ölü Atma Çukuru</t>
         </is>
       </c>
       <c r="C32" s="18" t="inlineStr">
         <is>
-          <t>TKDK-0042</t>
+          <t>15.160.1003</t>
         </is>
       </c>
       <c r="D32" s="16" t="inlineStr">
         <is>
-          <t>6 cm poliüretan dolgulu (üst min. 0,40 mm, alt min. 0,30 mm) boyalı galvanizli sac levhalar ile ısı yalıtımlı çatı kaplaması yapılması</t>
+          <t>Ø 8 - Ø 12 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
         </is>
       </c>
       <c r="E32" s="19" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>ton</t>
         </is>
       </c>
       <c r="F32" s="20" t="n">
-        <v>1204.98</v>
+        <v>1.657</v>
       </c>
       <c r="G32" s="5" t="n">
-        <v>1364.7228</v>
+        <v>39045.2412</v>
       </c>
       <c r="H32" s="5">
         <f>F32*G32</f>
         <v/>
       </c>
     </row>
-    <row r="33" ht="30" customHeight="1">
+    <row r="33" ht="20" customHeight="1">
       <c r="A33" s="16" t="inlineStr">
         <is>
-          <t>Çatı ve sundurma işleri</t>
+          <t>Demir-inşaat işleri</t>
         </is>
       </c>
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>Kümes B Blok</t>
+          <t>Foseptik</t>
         </is>
       </c>
       <c r="C33" s="18" t="inlineStr">
         <is>
-          <t>TKDK-0042</t>
+          <t>15.160.1003</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>6 cm poliüretan dolgulu (üst min. 0,40 mm, alt min. 0,30 mm) boyalı galvanizli sac levhalar ile ısı yalıtımlı çatı kaplaması yapılması</t>
+          <t>Ø 8 - Ø 12 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
         </is>
       </c>
       <c r="E33" s="19" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>ton</t>
         </is>
       </c>
       <c r="F33" s="20" t="n">
-        <v>1204.98</v>
+        <v>0.587</v>
       </c>
       <c r="G33" s="5" t="n">
-        <v>1364.7228</v>
+        <v>39045.2412</v>
       </c>
       <c r="H33" s="5">
         <f>F33*G33</f>
         <v/>
       </c>
     </row>
-    <row r="34" ht="14" customHeight="1">
+    <row r="34" ht="20" customHeight="1">
       <c r="A34" s="16" t="inlineStr">
         <is>
-          <t>Çevre düzenlemesi ve çit işleri</t>
+          <t>Demir-inşaat işleri</t>
         </is>
       </c>
       <c r="B34" s="17" t="inlineStr">
         <is>
-          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
+          <t>Yem Silosu Betonarme Kaideleri</t>
         </is>
       </c>
       <c r="C34" s="18" t="inlineStr">
         <is>
-          <t>TKDK-0091</t>
+          <t>15.160.1003</t>
         </is>
       </c>
       <c r="D34" s="16" t="inlineStr">
         <is>
-          <t>Betonarme direkli galvanizli tel örgü çit yapılması (Tip-1)</t>
+          <t>Ø 8 - Ø 12 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
         </is>
       </c>
       <c r="E34" s="19" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ton</t>
         </is>
       </c>
       <c r="F34" s="20" t="n">
-        <v>361.04</v>
+        <v>0.757</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>940.842</v>
+        <v>39045.2412</v>
       </c>
       <c r="H34" s="5">
         <f>F34*G34</f>
@@ -5940,96 +5940,96 @@
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="16" t="inlineStr">
         <is>
-          <t>Kanalizasyon işleri</t>
+          <t>Demir-inşaat işleri</t>
         </is>
       </c>
       <c r="B35" s="17" t="inlineStr">
         <is>
-          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
+          <t>Su Deposu</t>
         </is>
       </c>
       <c r="C35" s="18" t="inlineStr">
         <is>
-          <t>43.527.1001</t>
+          <t>15.160.1003</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>Çapı 150 mm HDPE koruge boru döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
+          <t>Ø 8 - Ø 12 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
         </is>
       </c>
       <c r="E35" s="19" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ton</t>
         </is>
       </c>
       <c r="F35" s="20" t="n">
-        <v>50</v>
+        <v>1.232</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>330.6996</v>
+        <v>39045.2412</v>
       </c>
       <c r="H35" s="5">
         <f>F35*G35</f>
         <v/>
       </c>
     </row>
-    <row r="36" ht="30" customHeight="1">
+    <row r="36" ht="20" customHeight="1">
       <c r="A36" s="16" t="inlineStr">
         <is>
-          <t>Betonarme işleri</t>
+          <t>Demir-inşaat işleri</t>
         </is>
       </c>
       <c r="B36" s="17" t="inlineStr">
         <is>
-          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
+          <t>Yağmur Suyu Deposu</t>
         </is>
       </c>
       <c r="C36" s="18" t="inlineStr">
         <is>
-          <t>15.150.1005</t>
+          <t>15.160.1003</t>
         </is>
       </c>
       <c r="D36" s="16" t="inlineStr">
         <is>
-          <t>Beton santralinde üretilen veya satın alınan ve beton pompasıyla basılan, C 25/30 basınç dayanım sınıfında, gri renkte, normal hazır beton dökülmesi (beton nakli dahil)</t>
+          <t>Ø 8 - Ø 12 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
         </is>
       </c>
       <c r="E36" s="19" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>ton</t>
         </is>
       </c>
       <c r="F36" s="20" t="n">
-        <v>1.566</v>
+        <v>1.23</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>2960.454</v>
+        <v>39045.2412</v>
       </c>
       <c r="H36" s="5">
         <f>F36*G36</f>
         <v/>
       </c>
     </row>
-    <row r="37" ht="14" customHeight="1">
+    <row r="37" ht="30" customHeight="1">
       <c r="A37" s="16" t="inlineStr">
         <is>
-          <t>Kalıp, yapı iskelesi işleri</t>
+          <t>Çatı ve sundurma işleri</t>
         </is>
       </c>
       <c r="B37" s="17" t="inlineStr">
         <is>
-          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
+          <t>Kümes A Blok</t>
         </is>
       </c>
       <c r="C37" s="18" t="inlineStr">
         <is>
-          <t>15.180.1003</t>
+          <t>TKDK-0042</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>Plywood ile düz yüzeyli betonarme kalıbı yapılması</t>
+          <t>6 cm poliüretan dolgulu (üst min. 0,40 mm, alt min. 0,30 mm) boyalı galvanizli sac levhalar ile ısı yalıtımlı çatı kaplaması yapılması</t>
         </is>
       </c>
       <c r="E37" s="19" t="inlineStr">
@@ -6038,47 +6038,47 @@
         </is>
       </c>
       <c r="F37" s="20" t="n">
-        <v>14.4</v>
+        <v>1204.98</v>
       </c>
       <c r="G37" s="5" t="n">
-        <v>863.7972</v>
+        <v>1364.7228</v>
       </c>
       <c r="H37" s="5">
         <f>F37*G37</f>
         <v/>
       </c>
     </row>
-    <row r="38" ht="20" customHeight="1">
+    <row r="38" ht="30" customHeight="1">
       <c r="A38" s="16" t="inlineStr">
         <is>
-          <t>Demir-inşaat işleri</t>
+          <t>Çatı ve sundurma işleri</t>
         </is>
       </c>
       <c r="B38" s="17" t="inlineStr">
         <is>
-          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
+          <t>Kümes B Blok</t>
         </is>
       </c>
       <c r="C38" s="18" t="inlineStr">
         <is>
-          <t>15.160.1003</t>
+          <t>TKDK-0042</t>
         </is>
       </c>
       <c r="D38" s="16" t="inlineStr">
         <is>
-          <t>Ø 8 - Ø 12 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
+          <t>6 cm poliüretan dolgulu (üst min. 0,40 mm, alt min. 0,30 mm) boyalı galvanizli sac levhalar ile ısı yalıtımlı çatı kaplaması yapılması</t>
         </is>
       </c>
       <c r="E38" s="19" t="inlineStr">
         <is>
-          <t>ton</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="F38" s="20" t="n">
-        <v>0.141</v>
+        <v>1204.98</v>
       </c>
       <c r="G38" s="5" t="n">
-        <v>39045.2412</v>
+        <v>1364.7228</v>
       </c>
       <c r="H38" s="5">
         <f>F38*G38</f>
@@ -6088,7 +6088,7 @@
     <row r="39" ht="14" customHeight="1">
       <c r="A39" s="16" t="inlineStr">
         <is>
-          <t>Kanalizasyon işleri</t>
+          <t>Çevre düzenlemesi ve çit işleri</t>
         </is>
       </c>
       <c r="B39" s="17" t="inlineStr">
@@ -6098,24 +6098,24 @@
       </c>
       <c r="C39" s="18" t="inlineStr">
         <is>
-          <t>15.560.1003</t>
+          <t>TKDK-0091</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>Betonarme kompozit rögar kapağı temini ve yerine konulması</t>
+          <t>Betonarme direkli galvanizli tel örgü çit yapılması (Tip-1)</t>
         </is>
       </c>
       <c r="E39" s="19" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="F39" s="20" t="n">
-        <v>4</v>
+        <v>361.04</v>
       </c>
       <c r="G39" s="5" t="n">
-        <v>3744.3</v>
+        <v>940.842</v>
       </c>
       <c r="H39" s="5">
         <f>F39*G39</f>
@@ -6125,7 +6125,7 @@
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="16" t="inlineStr">
         <is>
-          <t>Elektrik tesisatı ve aydınlatma</t>
+          <t>Kanalizasyon işleri</t>
         </is>
       </c>
       <c r="B40" s="17" t="inlineStr">
@@ -6135,34 +6135,34 @@
       </c>
       <c r="C40" s="18" t="inlineStr">
         <is>
-          <t>30.100.1104</t>
+          <t>43.527.1001</t>
         </is>
       </c>
       <c r="D40" s="16" t="inlineStr">
         <is>
-          <t>Ana dağıtım panosu (dikili tip galvanizli sac, en az 700 mm en, 400 mm derinlik)</t>
+          <t>Çapı 150 mm HDPE koruge boru döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
         </is>
       </c>
       <c r="E40" s="19" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="F40" s="20" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="G40" s="5" t="n">
-        <v>41783.1288</v>
+        <v>330.6996</v>
       </c>
       <c r="H40" s="5">
         <f>F40*G40</f>
         <v/>
       </c>
     </row>
-    <row r="41" ht="14" customHeight="1">
+    <row r="41" ht="30" customHeight="1">
       <c r="A41" s="16" t="inlineStr">
         <is>
-          <t>Elektrik tesisatı ve aydınlatma</t>
+          <t>Betonarme işleri</t>
         </is>
       </c>
       <c r="B41" s="17" t="inlineStr">
@@ -6172,34 +6172,34 @@
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>30.100.2106</t>
+          <t>15.150.1005</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>Sayaç panosu (sıva üstü galvanizli sac tablo, 0,50-0,60 m²)</t>
+          <t>Beton santralinde üretilen veya satın alınan ve beton pompasıyla basılan, C 25/30 basınç dayanım sınıfında, gri renkte, normal hazır beton dökülmesi (beton nakli dahil)</t>
         </is>
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="F41" s="20" t="n">
-        <v>1</v>
+        <v>1.566</v>
       </c>
       <c r="G41" s="5" t="n">
-        <v>11631.648</v>
+        <v>2960.454</v>
       </c>
       <c r="H41" s="5">
         <f>F41*G41</f>
         <v/>
       </c>
     </row>
-    <row r="42" ht="20" customHeight="1">
+    <row r="42" ht="14" customHeight="1">
       <c r="A42" s="16" t="inlineStr">
         <is>
-          <t>Elektrik tesisatı ve aydınlatma</t>
+          <t>Kalıp, yapı iskelesi işleri</t>
         </is>
       </c>
       <c r="B42" s="17" t="inlineStr">
@@ -6209,34 +6209,34 @@
       </c>
       <c r="C42" s="18" t="inlineStr">
         <is>
-          <t>30.135.3201</t>
+          <t>15.180.1003</t>
         </is>
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>Üç fazlı zaman tarifeli elektronik aktif sayaç, en az 5(100) A, 3x230/400 V</t>
+          <t>Plywood ile düz yüzeyli betonarme kalıbı yapılması</t>
         </is>
       </c>
       <c r="E42" s="19" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="F42" s="20" t="n">
-        <v>1</v>
+        <v>14.4</v>
       </c>
       <c r="G42" s="5" t="n">
-        <v>2218.1544</v>
+        <v>863.7972</v>
       </c>
       <c r="H42" s="5">
         <f>F42*G42</f>
         <v/>
       </c>
     </row>
-    <row r="43" ht="14" customHeight="1">
+    <row r="43" ht="20" customHeight="1">
       <c r="A43" s="16" t="inlineStr">
         <is>
-          <t>Elektrik tesisatı ve aydınlatma</t>
+          <t>Demir-inşaat işleri</t>
         </is>
       </c>
       <c r="B43" s="17" t="inlineStr">
@@ -6246,24 +6246,24 @@
       </c>
       <c r="C43" s="18" t="inlineStr">
         <is>
-          <t>30.110.1104</t>
+          <t>15.160.1003</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>Termik-manyetik kompakt şalter 3x160 A, Icu 35 kA — ana giriş</t>
+          <t>Ø 8 - Ø 12 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
         </is>
       </c>
       <c r="E43" s="19" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>ton</t>
         </is>
       </c>
       <c r="F43" s="20" t="n">
-        <v>1</v>
+        <v>0.141</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>5920.7568</v>
+        <v>39045.2412</v>
       </c>
       <c r="H43" s="5">
         <f>F43*G43</f>
@@ -6273,7 +6273,7 @@
     <row r="44" ht="14" customHeight="1">
       <c r="A44" s="16" t="inlineStr">
         <is>
-          <t>Elektrik tesisatı ve aydınlatma</t>
+          <t>Kanalizasyon işleri</t>
         </is>
       </c>
       <c r="B44" s="17" t="inlineStr">
@@ -6283,12 +6283,12 @@
       </c>
       <c r="C44" s="18" t="inlineStr">
         <is>
-          <t>30.115.1003</t>
+          <t>15.560.1003</t>
         </is>
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
-          <t>Kaçak akım koruma şalteri 2x63 A, 30 mA</t>
+          <t>Betonarme kompozit rögar kapağı temini ve yerine konulması</t>
         </is>
       </c>
       <c r="E44" s="19" t="inlineStr">
@@ -6297,10 +6297,10 @@
         </is>
       </c>
       <c r="F44" s="20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>1436.1984</v>
+        <v>3744.3</v>
       </c>
       <c r="H44" s="5">
         <f>F44*G44</f>
@@ -6320,31 +6320,31 @@
       </c>
       <c r="C45" s="18" t="inlineStr">
         <is>
-          <t>30.140.3105</t>
+          <t>30.100.1104</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>YVV (NYY) 1 kV yeraltı kablosu ile besleme hattı tesisi — 1x35 mm²</t>
+          <t>Ana dağıtım panosu (dikili tip galvanizli sac, en az 700 mm en, 400 mm derinlik)</t>
         </is>
       </c>
       <c r="E45" s="19" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="F45" s="20" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="G45" s="5" t="n">
-        <v>332.1696</v>
+        <v>41783.1288</v>
       </c>
       <c r="H45" s="5">
         <f>F45*G45</f>
         <v/>
       </c>
     </row>
-    <row r="46" ht="20" customHeight="1">
+    <row r="46" ht="14" customHeight="1">
       <c r="A46" s="16" t="inlineStr">
         <is>
           <t>Elektrik tesisatı ve aydınlatma</t>
@@ -6357,24 +6357,24 @@
       </c>
       <c r="C46" s="18" t="inlineStr">
         <is>
-          <t>30.140.3101</t>
+          <t>30.100.2106</t>
         </is>
       </c>
       <c r="D46" s="16" t="inlineStr">
         <is>
-          <t>YVV (NYY) 1 kV yeraltı kablosu ile besleme hattı tesisi — 1x6 mm²</t>
+          <t>Sayaç panosu (sıva üstü galvanizli sac tablo, 0,50-0,60 m²)</t>
         </is>
       </c>
       <c r="E46" s="19" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="F46" s="20" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>71.3244</v>
+        <v>11631.648</v>
       </c>
       <c r="H46" s="5">
         <f>F46*G46</f>
@@ -6394,12 +6394,12 @@
       </c>
       <c r="C47" s="18" t="inlineStr">
         <is>
-          <t>30.172.1706</t>
+          <t>30.135.3201</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>Aydınlatma direği — taban çapı en az 80 mm, yükseklik en az 4,00 m</t>
+          <t>Üç fazlı zaman tarifeli elektronik aktif sayaç, en az 5(100) A, 3x230/400 V</t>
         </is>
       </c>
       <c r="E47" s="19" t="inlineStr">
@@ -6408,10 +6408,10 @@
         </is>
       </c>
       <c r="F47" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>7783.1208</v>
+        <v>2218.1544</v>
       </c>
       <c r="H47" s="5">
         <f>F47*G47</f>
@@ -6431,12 +6431,12 @@
       </c>
       <c r="C48" s="18" t="inlineStr">
         <is>
-          <t>30.170.4002</t>
+          <t>30.110.1104</t>
         </is>
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>LED projektör, ışık akısı en az 5100 lm</t>
+          <t>Termik-manyetik kompakt şalter 3x160 A, Icu 35 kA — ana giriş</t>
         </is>
       </c>
       <c r="E48" s="19" t="inlineStr">
@@ -6445,10 +6445,10 @@
         </is>
       </c>
       <c r="F48" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>8313.1608</v>
+        <v>5920.7568</v>
       </c>
       <c r="H48" s="5">
         <f>F48*G48</f>
@@ -6463,17 +6463,17 @@
       </c>
       <c r="B49" s="17" t="inlineStr">
         <is>
-          <t>Kümes A Blok</t>
+          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
         </is>
       </c>
       <c r="C49" s="18" t="inlineStr">
         <is>
-          <t>30.120.2016</t>
+          <t>30.115.1003</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
-          <t>Otomatik transfer şalteri 4 x 200 A</t>
+          <t>Kaçak akım koruma şalteri 2x63 A, 30 mA</t>
         </is>
       </c>
       <c r="E49" s="19" t="inlineStr">
@@ -6482,17 +6482,17 @@
         </is>
       </c>
       <c r="F49" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G49" s="5" t="n">
-        <v>44709.8148</v>
+        <v>1436.1984</v>
       </c>
       <c r="H49" s="5">
         <f>F49*G49</f>
         <v/>
       </c>
     </row>
-    <row r="50" ht="14" customHeight="1">
+    <row r="50" ht="20" customHeight="1">
       <c r="A50" s="16" t="inlineStr">
         <is>
           <t>Elektrik tesisatı ve aydınlatma</t>
@@ -6500,49 +6500,234 @@
       </c>
       <c r="B50" s="17" t="inlineStr">
         <is>
-          <t>Kümes B Blok</t>
+          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
         </is>
       </c>
       <c r="C50" s="18" t="inlineStr">
         <is>
-          <t>30.120.2016</t>
+          <t>30.140.3105</t>
         </is>
       </c>
       <c r="D50" s="16" t="inlineStr">
         <is>
-          <t>Otomatik transfer şalteri 4 x 200 A</t>
+          <t>YVV (NYY) 1 kV yeraltı kablosu ile besleme hattı tesisi — 1x35 mm²</t>
         </is>
       </c>
       <c r="E50" s="19" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="F50" s="20" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="G50" s="5" t="n">
-        <v>44709.8148</v>
+        <v>332.1696</v>
       </c>
       <c r="H50" s="5">
         <f>F50*G50</f>
         <v/>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="21" t="n"/>
-      <c r="B51" s="21" t="n"/>
-      <c r="C51" s="21" t="n"/>
-      <c r="D51" s="22" t="inlineStr">
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="16" t="inlineStr">
+        <is>
+          <t>Elektrik tesisatı ve aydınlatma</t>
+        </is>
+      </c>
+      <c r="B51" s="17" t="inlineStr">
+        <is>
+          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>30.140.3101</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>YVV (NYY) 1 kV yeraltı kablosu ile besleme hattı tesisi — 1x6 mm²</t>
+        </is>
+      </c>
+      <c r="E51" s="19" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F51" s="20" t="n">
+        <v>50</v>
+      </c>
+      <c r="G51" s="5" t="n">
+        <v>71.3244</v>
+      </c>
+      <c r="H51" s="5">
+        <f>F51*G51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="16" t="inlineStr">
+        <is>
+          <t>Elektrik tesisatı ve aydınlatma</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
+        <is>
+          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>30.172.1706</t>
+        </is>
+      </c>
+      <c r="D52" s="16" t="inlineStr">
+        <is>
+          <t>Aydınlatma direği — taban çapı en az 80 mm, yükseklik en az 4,00 m</t>
+        </is>
+      </c>
+      <c r="E52" s="19" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="F52" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="G52" s="5" t="n">
+        <v>7783.1208</v>
+      </c>
+      <c r="H52" s="5">
+        <f>F52*G52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" ht="14" customHeight="1">
+      <c r="A53" s="16" t="inlineStr">
+        <is>
+          <t>Elektrik tesisatı ve aydınlatma</t>
+        </is>
+      </c>
+      <c r="B53" s="17" t="inlineStr">
+        <is>
+          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
+        </is>
+      </c>
+      <c r="C53" s="18" t="inlineStr">
+        <is>
+          <t>30.170.4002</t>
+        </is>
+      </c>
+      <c r="D53" s="16" t="inlineStr">
+        <is>
+          <t>LED projektör, ışık akısı en az 5100 lm</t>
+        </is>
+      </c>
+      <c r="E53" s="19" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="F53" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="G53" s="5" t="n">
+        <v>8313.1608</v>
+      </c>
+      <c r="H53" s="5">
+        <f>F53*G53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" ht="14" customHeight="1">
+      <c r="A54" s="16" t="inlineStr">
+        <is>
+          <t>Elektrik tesisatı ve aydınlatma</t>
+        </is>
+      </c>
+      <c r="B54" s="17" t="inlineStr">
+        <is>
+          <t>Kümes A Blok</t>
+        </is>
+      </c>
+      <c r="C54" s="18" t="inlineStr">
+        <is>
+          <t>30.120.2016</t>
+        </is>
+      </c>
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>Otomatik transfer şalteri 4 x 200 A</t>
+        </is>
+      </c>
+      <c r="E54" s="19" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="F54" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="5" t="n">
+        <v>44709.8148</v>
+      </c>
+      <c r="H54" s="5">
+        <f>F54*G54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="14" customHeight="1">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
+          <t>Elektrik tesisatı ve aydınlatma</t>
+        </is>
+      </c>
+      <c r="B55" s="17" t="inlineStr">
+        <is>
+          <t>Kümes B Blok</t>
+        </is>
+      </c>
+      <c r="C55" s="18" t="inlineStr">
+        <is>
+          <t>30.120.2016</t>
+        </is>
+      </c>
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>Otomatik transfer şalteri 4 x 200 A</t>
+        </is>
+      </c>
+      <c r="E55" s="19" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="F55" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="5" t="n">
+        <v>44709.8148</v>
+      </c>
+      <c r="H55" s="5">
+        <f>F55*G55</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="21" t="n"/>
+      <c r="B56" s="21" t="n"/>
+      <c r="C56" s="21" t="n"/>
+      <c r="D56" s="22" t="inlineStr">
         <is>
           <t>HİBE DIŞI YAPIM İŞLERİ TOPLAMI (KDV hariç)</t>
         </is>
       </c>
-      <c r="E51" s="21" t="n"/>
-      <c r="F51" s="21" t="n"/>
-      <c r="G51" s="21" t="n"/>
-      <c r="H51" s="9">
-        <f>SUM(H5:H50)</f>
+      <c r="E56" s="21" t="n"/>
+      <c r="F56" s="21" t="n"/>
+      <c r="G56" s="21" t="n"/>
+      <c r="H56" s="9">
+        <f>SUM(H5:H55)</f>
         <v/>
       </c>
     </row>
@@ -6915,7 +7100,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>24879695.26</v>
+        <v>24817978.39</v>
       </c>
       <c r="C5" s="6">
         <f>B5/52.7585</f>
@@ -6953,7 +7138,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>5497755.42</v>
+        <v>5659298.55</v>
       </c>
       <c r="C7" s="6">
         <f>B7/52.7585</f>
@@ -6972,7 +7157,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>3095220</v>
+        <v>2871960</v>
       </c>
       <c r="C8" s="6">
         <f>B8/52.7585</f>
@@ -7010,7 +7195,7 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>9302975.42</v>
+        <v>9241258.550000001</v>
       </c>
       <c r="C10" s="10">
         <f>B10/52.7585</f>
@@ -7048,7 +7233,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>4975939.05</v>
+        <v>4963595.68</v>
       </c>
       <c r="C12" s="6">
         <f>B12/52.7585</f>

</xml_diff>

<commit_message>
Yayın: hibe dışı proforma kitap fiyatına geçti
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
+++ b/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
@@ -4780,7 +4780,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Kümes A ve B blokları dışındaki yapılar ile bu iki bloktan hibe kapsamı dışına çıkarılan pozlar. Bu imalatlar yapılmaya devam eder; teklif alma usulüne tabi değildir, proforma fatura ile beyan edilir ve tamamı öz kaynaktan karşılanır.</t>
+          <t>Kümes A ve B blokları dışındaki yapılar ile bu iki bloktan hibe kapsamı dışına çıkarılan pozlar. Bu imalatlar yapılmaya devam eder; teklif alma usulüne tabi değildir, proforma fatura ile beyan edilir ve tamamı öz kaynaktan karşılanır. Birim fiyatlar kitabın kendi fiyatlarıdır; %16 tenzilat uygulanmaz, çünkü tenzilat idarenin yaklaşık maliyet beklentisidir, satıcının fiyatı değildir.</t>
         </is>
       </c>
     </row>
@@ -4857,7 +4857,7 @@
         <v>260.942</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>52.374</v>
+        <v>62.35</v>
       </c>
       <c r="H5" s="5">
         <f>F5*G5</f>
@@ -4894,7 +4894,7 @@
         <v>542.7</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>60.354</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="H6" s="5">
         <f>F6*G6</f>
@@ -4931,7 +4931,7 @@
         <v>142</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>60.354</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="H7" s="5">
         <f>F7*G7</f>
@@ -4968,7 +4968,7 @@
         <v>48.8</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>60.354</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="H8" s="5">
         <f>F8*G8</f>
@@ -5005,7 +5005,7 @@
         <v>48.02</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>60.354</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="H9" s="5">
         <f>F9*G9</f>
@@ -5042,7 +5042,7 @@
         <v>106.5</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>60.354</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="H10" s="5">
         <f>F10*G10</f>
@@ -5079,7 +5079,7 @@
         <v>88.75</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>60.354</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="H11" s="5">
         <f>F11*G11</f>
@@ -5116,7 +5116,7 @@
         <v>11.934</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>2750.454</v>
+        <v>3274.35</v>
       </c>
       <c r="H12" s="5">
         <f>F12*G12</f>
@@ -5153,7 +5153,7 @@
         <v>1.984</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>2750.454</v>
+        <v>3274.35</v>
       </c>
       <c r="H13" s="5">
         <f>F13*G13</f>
@@ -5190,7 +5190,7 @@
         <v>0.484</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>2750.454</v>
+        <v>3274.35</v>
       </c>
       <c r="H14" s="5">
         <f>F14*G14</f>
@@ -5227,7 +5227,7 @@
         <v>1.922</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>2750.454</v>
+        <v>3274.35</v>
       </c>
       <c r="H15" s="5">
         <f>F15*G15</f>
@@ -5264,7 +5264,7 @@
         <v>1.344</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>2750.454</v>
+        <v>3274.35</v>
       </c>
       <c r="H16" s="5">
         <f>F16*G16</f>
@@ -5301,7 +5301,7 @@
         <v>1.024</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>2750.454</v>
+        <v>3274.35</v>
       </c>
       <c r="H17" s="5">
         <f>F17*G17</f>
@@ -5338,7 +5338,7 @@
         <v>93.19</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>2960.454</v>
+        <v>3524.35</v>
       </c>
       <c r="H18" s="5">
         <f>F18*G18</f>
@@ -5375,7 +5375,7 @@
         <v>20.85</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>2960.454</v>
+        <v>3524.35</v>
       </c>
       <c r="H19" s="5">
         <f>F19*G19</f>
@@ -5412,7 +5412,7 @@
         <v>15.15</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>2960.454</v>
+        <v>3524.35</v>
       </c>
       <c r="H20" s="5">
         <f>F20*G20</f>
@@ -5449,7 +5449,7 @@
         <v>12.3</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>2960.454</v>
+        <v>3524.35</v>
       </c>
       <c r="H21" s="5">
         <f>F21*G21</f>
@@ -5486,7 +5486,7 @@
         <v>6.175</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>2960.454</v>
+        <v>3524.35</v>
       </c>
       <c r="H22" s="5">
         <f>F22*G22</f>
@@ -5523,7 +5523,7 @@
         <v>8.41</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>2960.454</v>
+        <v>3524.35</v>
       </c>
       <c r="H23" s="5">
         <f>F23*G23</f>
@@ -5560,7 +5560,7 @@
         <v>363.26</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>863.7972</v>
+        <v>1028.33</v>
       </c>
       <c r="H24" s="5">
         <f>F24*G24</f>
@@ -5597,7 +5597,7 @@
         <v>127.2</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>863.7972</v>
+        <v>1028.33</v>
       </c>
       <c r="H25" s="5">
         <f>F25*G25</f>
@@ -5634,7 +5634,7 @@
         <v>95.59999999999999</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>863.7972</v>
+        <v>1028.33</v>
       </c>
       <c r="H26" s="5">
         <f>F26*G26</f>
@@ -5671,7 +5671,7 @@
         <v>79.8</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>863.7972</v>
+        <v>1028.33</v>
       </c>
       <c r="H27" s="5">
         <f>F27*G27</f>
@@ -5708,7 +5708,7 @@
         <v>41.4</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>863.7972</v>
+        <v>1028.33</v>
       </c>
       <c r="H28" s="5">
         <f>F28*G28</f>
@@ -5745,7 +5745,7 @@
         <v>11.6</v>
       </c>
       <c r="G29" s="5" t="n">
-        <v>863.7972</v>
+        <v>1028.33</v>
       </c>
       <c r="H29" s="5">
         <f>F29*G29</f>
@@ -5782,7 +5782,7 @@
         <v>7.599</v>
       </c>
       <c r="G30" s="5" t="n">
-        <v>39045.2412</v>
+        <v>46482.43</v>
       </c>
       <c r="H30" s="5">
         <f>F30*G30</f>
@@ -5819,7 +5819,7 @@
         <v>0.5639999999999999</v>
       </c>
       <c r="G31" s="5" t="n">
-        <v>37532.1912</v>
+        <v>44681.18</v>
       </c>
       <c r="H31" s="5">
         <f>F31*G31</f>
@@ -5856,7 +5856,7 @@
         <v>1.657</v>
       </c>
       <c r="G32" s="5" t="n">
-        <v>39045.2412</v>
+        <v>46482.43</v>
       </c>
       <c r="H32" s="5">
         <f>F32*G32</f>
@@ -5893,7 +5893,7 @@
         <v>0.587</v>
       </c>
       <c r="G33" s="5" t="n">
-        <v>39045.2412</v>
+        <v>46482.43</v>
       </c>
       <c r="H33" s="5">
         <f>F33*G33</f>
@@ -5930,7 +5930,7 @@
         <v>0.757</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>39045.2412</v>
+        <v>46482.43</v>
       </c>
       <c r="H34" s="5">
         <f>F34*G34</f>
@@ -5967,7 +5967,7 @@
         <v>1.232</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>39045.2412</v>
+        <v>46482.43</v>
       </c>
       <c r="H35" s="5">
         <f>F35*G35</f>
@@ -6004,7 +6004,7 @@
         <v>1.23</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>39045.2412</v>
+        <v>46482.43</v>
       </c>
       <c r="H36" s="5">
         <f>F36*G36</f>
@@ -6041,7 +6041,7 @@
         <v>1204.98</v>
       </c>
       <c r="G37" s="5" t="n">
-        <v>1364.7228</v>
+        <v>1624.67</v>
       </c>
       <c r="H37" s="5">
         <f>F37*G37</f>
@@ -6078,7 +6078,7 @@
         <v>1204.98</v>
       </c>
       <c r="G38" s="5" t="n">
-        <v>1364.7228</v>
+        <v>1624.67</v>
       </c>
       <c r="H38" s="5">
         <f>F38*G38</f>
@@ -6115,7 +6115,7 @@
         <v>361.04</v>
       </c>
       <c r="G39" s="5" t="n">
-        <v>940.842</v>
+        <v>1120.05</v>
       </c>
       <c r="H39" s="5">
         <f>F39*G39</f>
@@ -6152,7 +6152,7 @@
         <v>50</v>
       </c>
       <c r="G40" s="5" t="n">
-        <v>330.6996</v>
+        <v>393.69</v>
       </c>
       <c r="H40" s="5">
         <f>F40*G40</f>
@@ -6189,7 +6189,7 @@
         <v>1.566</v>
       </c>
       <c r="G41" s="5" t="n">
-        <v>2960.454</v>
+        <v>3524.35</v>
       </c>
       <c r="H41" s="5">
         <f>F41*G41</f>
@@ -6226,7 +6226,7 @@
         <v>14.4</v>
       </c>
       <c r="G42" s="5" t="n">
-        <v>863.7972</v>
+        <v>1028.33</v>
       </c>
       <c r="H42" s="5">
         <f>F42*G42</f>
@@ -6263,7 +6263,7 @@
         <v>0.141</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>39045.2412</v>
+        <v>46482.43</v>
       </c>
       <c r="H43" s="5">
         <f>F43*G43</f>
@@ -6300,7 +6300,7 @@
         <v>4</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>3744.3</v>
+        <v>4457.5</v>
       </c>
       <c r="H44" s="5">
         <f>F44*G44</f>
@@ -6337,7 +6337,7 @@
         <v>1</v>
       </c>
       <c r="G45" s="5" t="n">
-        <v>31602.3288</v>
+        <v>37621.82</v>
       </c>
       <c r="H45" s="5">
         <f>F45*G45</f>
@@ -6374,7 +6374,7 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>8179.248</v>
+        <v>9737.200000000001</v>
       </c>
       <c r="H46" s="5">
         <f>F46*G46</f>
@@ -6411,7 +6411,7 @@
         <v>1</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>1504.1544</v>
+        <v>1790.66</v>
       </c>
       <c r="H47" s="5">
         <f>F47*G47</f>
@@ -6448,7 +6448,7 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>4753.1568</v>
+        <v>5658.52</v>
       </c>
       <c r="H48" s="5">
         <f>F48*G48</f>
@@ -6485,7 +6485,7 @@
         <v>2</v>
       </c>
       <c r="G49" s="5" t="n">
-        <v>1079.1984</v>
+        <v>1284.76</v>
       </c>
       <c r="H49" s="5">
         <f>F49*G49</f>
@@ -6522,7 +6522,7 @@
         <v>50</v>
       </c>
       <c r="G50" s="5" t="n">
-        <v>277.1496</v>
+        <v>329.94</v>
       </c>
       <c r="H50" s="5">
         <f>F50*G50</f>
@@ -6559,7 +6559,7 @@
         <v>50</v>
       </c>
       <c r="G51" s="5" t="n">
-        <v>51.2484</v>
+        <v>61.01</v>
       </c>
       <c r="H51" s="5">
         <f>F51*G51</f>
@@ -6596,7 +6596,7 @@
         <v>4</v>
       </c>
       <c r="G52" s="5" t="n">
-        <v>6229.1208</v>
+        <v>7415.62</v>
       </c>
       <c r="H52" s="5">
         <f>F52*G52</f>
@@ -6633,7 +6633,7 @@
         <v>4</v>
       </c>
       <c r="G53" s="5" t="n">
-        <v>7632.7608</v>
+        <v>9086.620000000001</v>
       </c>
       <c r="H53" s="5">
         <f>F53*G53</f>
@@ -6670,7 +6670,7 @@
         <v>1</v>
       </c>
       <c r="G54" s="5" t="n">
-        <v>38544.2148</v>
+        <v>45885.97</v>
       </c>
       <c r="H54" s="5">
         <f>F54*G54</f>
@@ -6707,7 +6707,7 @@
         <v>1</v>
       </c>
       <c r="G55" s="5" t="n">
-        <v>38544.2148</v>
+        <v>45885.97</v>
       </c>
       <c r="H55" s="5">
         <f>F55*G55</f>
@@ -7100,7 +7100,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>24545301.31</v>
+        <v>25615426.2</v>
       </c>
       <c r="C5" s="6">
         <f>B5/52.7585</f>
@@ -7138,7 +7138,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>5618046.15</v>
+        <v>6688171.04</v>
       </c>
       <c r="C7" s="6">
         <f>B7/52.7585</f>
@@ -7195,7 +7195,7 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>9200006.15</v>
+        <v>10270131.04</v>
       </c>
       <c r="C10" s="10">
         <f>B10/52.7585</f>
@@ -7233,7 +7233,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>4909060.26</v>
+        <v>5123085.24</v>
       </c>
       <c r="C12" s="6">
         <f>B12/52.7585</f>

</xml_diff>

<commit_message>
Yayın: hibe dışı proforma %16 tenzilatlı fiyata döndü
Proforma 36 ve A3.4-EK Yapım sayfası tenzilatlı birim fiyata döndü;
hibe dışı yapım işleri 6.688.171,04 TL'den 5.618.052,70 TL'ye indi.
Uygun harcama, hibe tutarı ve kriter 1 payı değişmedi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
+++ b/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
@@ -4780,7 +4780,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Kümes A ve B blokları dışındaki yapılar ile bu iki bloktan hibe kapsamı dışına çıkarılan pozlar. Bu imalatlar yapılmaya devam eder; teklif alma usulüne tabi değildir, proforma fatura ile beyan edilir ve tamamı öz kaynaktan karşılanır. Birim fiyatlar kitabın kendi fiyatlarıdır; %16 tenzilat uygulanmaz, çünkü tenzilat idarenin yaklaşık maliyet beklentisidir, satıcının fiyatı değildir.</t>
+          <t>Kümes A ve B blokları dışındaki yapılar ile bu iki bloktan hibe kapsamı dışına çıkarılan pozlar. Bu imalatlar yapılmaya devam eder; teklif alma usulüne tabi değildir, proforma fatura ile beyan edilir ve tamamı öz kaynaktan karşılanır. Birim fiyatlar, hibe kapsamındaki işlerle aynı esasa göre kurulmuştur: ÇŞB 2026 ve TKDK 17.02.2026 kitap fiyatlarına %16 tenzilat uygulanmıştır.</t>
         </is>
       </c>
     </row>
@@ -4857,7 +4857,7 @@
         <v>260.942</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>62.35</v>
+        <v>52.37</v>
       </c>
       <c r="H5" s="5">
         <f>F5*G5</f>
@@ -4894,7 +4894,7 @@
         <v>542.7</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>71.84999999999999</v>
+        <v>60.35</v>
       </c>
       <c r="H6" s="5">
         <f>F6*G6</f>
@@ -4931,7 +4931,7 @@
         <v>142</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>71.84999999999999</v>
+        <v>60.35</v>
       </c>
       <c r="H7" s="5">
         <f>F7*G7</f>
@@ -4968,7 +4968,7 @@
         <v>48.8</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>71.84999999999999</v>
+        <v>60.35</v>
       </c>
       <c r="H8" s="5">
         <f>F8*G8</f>
@@ -5005,7 +5005,7 @@
         <v>48.02</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>71.84999999999999</v>
+        <v>60.35</v>
       </c>
       <c r="H9" s="5">
         <f>F9*G9</f>
@@ -5042,7 +5042,7 @@
         <v>106.5</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>71.84999999999999</v>
+        <v>60.35</v>
       </c>
       <c r="H10" s="5">
         <f>F10*G10</f>
@@ -5079,7 +5079,7 @@
         <v>88.75</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>71.84999999999999</v>
+        <v>60.35</v>
       </c>
       <c r="H11" s="5">
         <f>F11*G11</f>
@@ -5116,7 +5116,7 @@
         <v>11.934</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>3274.35</v>
+        <v>2750.45</v>
       </c>
       <c r="H12" s="5">
         <f>F12*G12</f>
@@ -5153,7 +5153,7 @@
         <v>1.984</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>3274.35</v>
+        <v>2750.45</v>
       </c>
       <c r="H13" s="5">
         <f>F13*G13</f>
@@ -5190,7 +5190,7 @@
         <v>0.484</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>3274.35</v>
+        <v>2750.45</v>
       </c>
       <c r="H14" s="5">
         <f>F14*G14</f>
@@ -5227,7 +5227,7 @@
         <v>1.922</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>3274.35</v>
+        <v>2750.45</v>
       </c>
       <c r="H15" s="5">
         <f>F15*G15</f>
@@ -5264,7 +5264,7 @@
         <v>1.344</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>3274.35</v>
+        <v>2750.45</v>
       </c>
       <c r="H16" s="5">
         <f>F16*G16</f>
@@ -5301,7 +5301,7 @@
         <v>1.024</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>3274.35</v>
+        <v>2750.45</v>
       </c>
       <c r="H17" s="5">
         <f>F17*G17</f>
@@ -5338,7 +5338,7 @@
         <v>93.19</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>3524.35</v>
+        <v>2960.45</v>
       </c>
       <c r="H18" s="5">
         <f>F18*G18</f>
@@ -5375,7 +5375,7 @@
         <v>20.85</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>3524.35</v>
+        <v>2960.45</v>
       </c>
       <c r="H19" s="5">
         <f>F19*G19</f>
@@ -5412,7 +5412,7 @@
         <v>15.15</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>3524.35</v>
+        <v>2960.45</v>
       </c>
       <c r="H20" s="5">
         <f>F20*G20</f>
@@ -5449,7 +5449,7 @@
         <v>12.3</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>3524.35</v>
+        <v>2960.45</v>
       </c>
       <c r="H21" s="5">
         <f>F21*G21</f>
@@ -5486,7 +5486,7 @@
         <v>6.175</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>3524.35</v>
+        <v>2960.45</v>
       </c>
       <c r="H22" s="5">
         <f>F22*G22</f>
@@ -5523,7 +5523,7 @@
         <v>8.41</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>3524.35</v>
+        <v>2960.45</v>
       </c>
       <c r="H23" s="5">
         <f>F23*G23</f>
@@ -5560,7 +5560,7 @@
         <v>363.26</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>1028.33</v>
+        <v>863.8</v>
       </c>
       <c r="H24" s="5">
         <f>F24*G24</f>
@@ -5597,7 +5597,7 @@
         <v>127.2</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>1028.33</v>
+        <v>863.8</v>
       </c>
       <c r="H25" s="5">
         <f>F25*G25</f>
@@ -5634,7 +5634,7 @@
         <v>95.59999999999999</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>1028.33</v>
+        <v>863.8</v>
       </c>
       <c r="H26" s="5">
         <f>F26*G26</f>
@@ -5671,7 +5671,7 @@
         <v>79.8</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>1028.33</v>
+        <v>863.8</v>
       </c>
       <c r="H27" s="5">
         <f>F27*G27</f>
@@ -5708,7 +5708,7 @@
         <v>41.4</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>1028.33</v>
+        <v>863.8</v>
       </c>
       <c r="H28" s="5">
         <f>F28*G28</f>
@@ -5745,7 +5745,7 @@
         <v>11.6</v>
       </c>
       <c r="G29" s="5" t="n">
-        <v>1028.33</v>
+        <v>863.8</v>
       </c>
       <c r="H29" s="5">
         <f>F29*G29</f>
@@ -5782,7 +5782,7 @@
         <v>7.599</v>
       </c>
       <c r="G30" s="5" t="n">
-        <v>46482.43</v>
+        <v>39045.24</v>
       </c>
       <c r="H30" s="5">
         <f>F30*G30</f>
@@ -5819,7 +5819,7 @@
         <v>0.5639999999999999</v>
       </c>
       <c r="G31" s="5" t="n">
-        <v>44681.18</v>
+        <v>37532.19</v>
       </c>
       <c r="H31" s="5">
         <f>F31*G31</f>
@@ -5856,7 +5856,7 @@
         <v>1.657</v>
       </c>
       <c r="G32" s="5" t="n">
-        <v>46482.43</v>
+        <v>39045.24</v>
       </c>
       <c r="H32" s="5">
         <f>F32*G32</f>
@@ -5893,7 +5893,7 @@
         <v>0.587</v>
       </c>
       <c r="G33" s="5" t="n">
-        <v>46482.43</v>
+        <v>39045.24</v>
       </c>
       <c r="H33" s="5">
         <f>F33*G33</f>
@@ -5930,7 +5930,7 @@
         <v>0.757</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>46482.43</v>
+        <v>39045.24</v>
       </c>
       <c r="H34" s="5">
         <f>F34*G34</f>
@@ -5967,7 +5967,7 @@
         <v>1.232</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>46482.43</v>
+        <v>39045.24</v>
       </c>
       <c r="H35" s="5">
         <f>F35*G35</f>
@@ -6004,7 +6004,7 @@
         <v>1.23</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>46482.43</v>
+        <v>39045.24</v>
       </c>
       <c r="H36" s="5">
         <f>F36*G36</f>
@@ -6041,7 +6041,7 @@
         <v>1204.98</v>
       </c>
       <c r="G37" s="5" t="n">
-        <v>1624.67</v>
+        <v>1364.72</v>
       </c>
       <c r="H37" s="5">
         <f>F37*G37</f>
@@ -6078,7 +6078,7 @@
         <v>1204.98</v>
       </c>
       <c r="G38" s="5" t="n">
-        <v>1624.67</v>
+        <v>1364.72</v>
       </c>
       <c r="H38" s="5">
         <f>F38*G38</f>
@@ -6115,7 +6115,7 @@
         <v>361.04</v>
       </c>
       <c r="G39" s="5" t="n">
-        <v>1120.05</v>
+        <v>940.84</v>
       </c>
       <c r="H39" s="5">
         <f>F39*G39</f>
@@ -6152,7 +6152,7 @@
         <v>50</v>
       </c>
       <c r="G40" s="5" t="n">
-        <v>393.69</v>
+        <v>330.7</v>
       </c>
       <c r="H40" s="5">
         <f>F40*G40</f>
@@ -6189,7 +6189,7 @@
         <v>1.566</v>
       </c>
       <c r="G41" s="5" t="n">
-        <v>3524.35</v>
+        <v>2960.45</v>
       </c>
       <c r="H41" s="5">
         <f>F41*G41</f>
@@ -6226,7 +6226,7 @@
         <v>14.4</v>
       </c>
       <c r="G42" s="5" t="n">
-        <v>1028.33</v>
+        <v>863.8</v>
       </c>
       <c r="H42" s="5">
         <f>F42*G42</f>
@@ -6263,7 +6263,7 @@
         <v>0.141</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>46482.43</v>
+        <v>39045.24</v>
       </c>
       <c r="H43" s="5">
         <f>F43*G43</f>
@@ -6300,7 +6300,7 @@
         <v>4</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>4457.5</v>
+        <v>3744.3</v>
       </c>
       <c r="H44" s="5">
         <f>F44*G44</f>
@@ -6337,7 +6337,7 @@
         <v>1</v>
       </c>
       <c r="G45" s="5" t="n">
-        <v>37621.82</v>
+        <v>31602.33</v>
       </c>
       <c r="H45" s="5">
         <f>F45*G45</f>
@@ -6374,7 +6374,7 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>9737.200000000001</v>
+        <v>8179.25</v>
       </c>
       <c r="H46" s="5">
         <f>F46*G46</f>
@@ -6411,7 +6411,7 @@
         <v>1</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>1790.66</v>
+        <v>1504.15</v>
       </c>
       <c r="H47" s="5">
         <f>F47*G47</f>
@@ -6448,7 +6448,7 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>5658.52</v>
+        <v>4753.16</v>
       </c>
       <c r="H48" s="5">
         <f>F48*G48</f>
@@ -6485,7 +6485,7 @@
         <v>2</v>
       </c>
       <c r="G49" s="5" t="n">
-        <v>1284.76</v>
+        <v>1079.2</v>
       </c>
       <c r="H49" s="5">
         <f>F49*G49</f>
@@ -6522,7 +6522,7 @@
         <v>50</v>
       </c>
       <c r="G50" s="5" t="n">
-        <v>329.94</v>
+        <v>277.15</v>
       </c>
       <c r="H50" s="5">
         <f>F50*G50</f>
@@ -6559,7 +6559,7 @@
         <v>50</v>
       </c>
       <c r="G51" s="5" t="n">
-        <v>61.01</v>
+        <v>51.25</v>
       </c>
       <c r="H51" s="5">
         <f>F51*G51</f>
@@ -6596,7 +6596,7 @@
         <v>4</v>
       </c>
       <c r="G52" s="5" t="n">
-        <v>7415.62</v>
+        <v>6229.12</v>
       </c>
       <c r="H52" s="5">
         <f>F52*G52</f>
@@ -6633,7 +6633,7 @@
         <v>4</v>
       </c>
       <c r="G53" s="5" t="n">
-        <v>9086.620000000001</v>
+        <v>7632.76</v>
       </c>
       <c r="H53" s="5">
         <f>F53*G53</f>
@@ -6670,7 +6670,7 @@
         <v>1</v>
       </c>
       <c r="G54" s="5" t="n">
-        <v>45885.97</v>
+        <v>38544.21</v>
       </c>
       <c r="H54" s="5">
         <f>F54*G54</f>
@@ -6707,7 +6707,7 @@
         <v>1</v>
       </c>
       <c r="G55" s="5" t="n">
-        <v>45885.97</v>
+        <v>38544.21</v>
       </c>
       <c r="H55" s="5">
         <f>F55*G55</f>
@@ -7100,7 +7100,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>25615426.2</v>
+        <v>24545307.86</v>
       </c>
       <c r="C5" s="6">
         <f>B5/52.7585</f>
@@ -7138,7 +7138,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>6688171.04</v>
+        <v>5618052.7</v>
       </c>
       <c r="C7" s="6">
         <f>B7/52.7585</f>
@@ -7195,7 +7195,7 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>10270131.04</v>
+        <v>9200012.699999999</v>
       </c>
       <c r="C10" s="10">
         <f>B10/52.7585</f>
@@ -7233,7 +7233,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>5123085.24</v>
+        <v>4909061.57</v>
       </c>
       <c r="C12" s="6">
         <f>B12/52.7585</f>

</xml_diff>

<commit_message>
IPARD paketi: Teknik Proje (TP 101-3) ve B2 Is Plani eklendi
Yayin sayfasina 44_TEKNIK_PROJE_TP1013.xlsx ve 45_B2_IS_PLANI.pdf girdi
(56 belge). Makine-ekipman ihtiyac listesi tedarikci teknik sartnamesine
oturtuldu; isitma sistemi kendi lotundaki gercek teklifiyle durur.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
+++ b/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>'A3.4-EK Makine-Ekipman'!G21</f>
+        <f>'A3.4-EK Makine-Ekipman'!G13</f>
         <v/>
       </c>
       <c r="C13" s="6">
@@ -4257,15 +4257,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -4297,22 +4297,22 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Ürün adı</t>
+          <t>Ürün kodu</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Birim</t>
+          <t>Makine-ekipmanın adı ve teknik özeti</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Miktar</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Birim fiyat (TL)</t>
+          <t>Bina başına (TL)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -4321,7 +4321,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Makine ve ekipman alımı</t>
@@ -4330,28 +4330,28 @@
       <c r="B5" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>Yemlik depo motor grubu (170 kg yem deposu, milli yemlik motoru, yemlik hat sonu, elektrik kutusu ile)</t>
-        </is>
-      </c>
-      <c r="D5" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E5" s="20" t="n">
-        <v>6</v>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>HZC-FD-01</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Yemleme sistemi — 3 hat, 243 m hat uzunluğu, 150 kg galvanizli yem deposu x 3, 0,55 kW yemlik motoru x 3, 35 cm çapında 324 plastik yemlik, 1,1 kW çift redüktörlü frenli otomatik kaldırma</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>2</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>22000</v>
+        <v>250062.04</v>
       </c>
       <c r="G5" s="5">
         <f>ROUND(E5*F5,2)</f>
         <v/>
       </c>
     </row>
-    <row r="6" ht="14" customHeight="1">
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Makine ve ekipman alımı</t>
@@ -4360,21 +4360,21 @@
       <c r="B6" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>Spiral yemleme sistemi (yemlik boru, yemlik tabağı, yay, boru kelepçesi)</t>
-        </is>
-      </c>
-      <c r="D6" s="19" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="E6" s="20" t="n">
-        <v>468</v>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>HZC-COM-004</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>Kümes kontrol panosu — HZC-70 işlemcili; 5 sıcaklık, 1 nem, 1 basınç ve 1 CO2 sensörü, alarm sistemi, uzaktan erişim, PLC kontrol, raporlama ve analiz</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>2</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>510</v>
+        <v>262674.92</v>
       </c>
       <c r="G6" s="5">
         <f>ROUND(E6*F6,2)</f>
@@ -4390,28 +4390,28 @@
       <c r="B7" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>15'li nipel sulama sistemi (20 cm'de bir krom nipelli boru, nipel çanağı, muf ve muf teli ile)</t>
-        </is>
-      </c>
-      <c r="D7" s="19" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="E7" s="20" t="n">
-        <v>624</v>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>HZC-WNT-012</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Tünel havalandırma fanı — 4 adet, 138 x 138 x 42 cm, 40.000 m³/h, 1,5 kW, galvanizli çelik kanat, ahtapot sistemli otomatik panjur</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>2</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>285</v>
+        <v>76982.48</v>
       </c>
       <c r="G7" s="5">
         <f>ROUND(E7*F7,2)</f>
         <v/>
       </c>
     </row>
-    <row r="8" ht="14" customHeight="1">
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Makine ve ekipman alımı</t>
@@ -4420,28 +4420,28 @@
       <c r="B8" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>Regülatör takımı</t>
-        </is>
-      </c>
-      <c r="D8" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E8" s="20" t="n">
-        <v>8</v>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>HZC-WTR-005</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Sulama sistemi — 4 hat, hat başına 312 m, 22 x 22 mm hat çapı, 1.560 metal 360° nipel suluk, 4 regülatör, 0,75 kW çift redüktörlü frenli otomatik kaldırma</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>2</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>1800</v>
+        <v>145353.3</v>
       </c>
       <c r="G8" s="5">
         <f>ROUND(E8*F8,2)</f>
         <v/>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1">
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Makine ve ekipman alımı</t>
@@ -4450,21 +4450,21 @@
       <c r="B9" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="16" t="inlineStr">
-        <is>
-          <t>Yemlik ve suluk kaldırma sistemi (6 ve 5 mm halat, sarı ve beyaz ip, klemens, plastik makara, askı saçı, bilyalı makara)</t>
-        </is>
-      </c>
-      <c r="D9" s="19" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="E9" s="20" t="n">
-        <v>1260</v>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>HZC-WNT-024</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Soğutma pedi sistemi — Tüplü, dahili devridaimli; 15 cm kalınlık, 150 cm yükseklik, 2 x 15 m uzunluk (45 m² ped alanı), PVC çerçeve, XPS petek kapakları, 2 aktüatör, 2 adet 0,50 kW su pompası</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>2</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>55</v>
+        <v>269272.63</v>
       </c>
       <c r="G9" s="5">
         <f>ROUND(E9*F9,2)</f>
@@ -4480,21 +4480,21 @@
       <c r="B10" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="C10" s="16" t="inlineStr">
-        <is>
-          <t>Yemlik motorlu kaldırma sistemi (1,1 kW çift redüktörlü frenli kaldırma motoru, mafsal 50'lik boru, UCP bilya, kontrol panosu dâhil)</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E10" s="20" t="n">
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>HZC-WNT-001</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>Klape sistemi — 40 adet 26 x 56 cm izolasyonlu plastik klape, klape başına 1.750 m³/h, 2 aktüatörlü açma-kapama, 161 m hat</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>50000</v>
+        <v>40581.31</v>
       </c>
       <c r="G10" s="5">
         <f>ROUND(E10*F10,2)</f>
@@ -4510,21 +4510,21 @@
       <c r="B11" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="C11" s="16" t="inlineStr">
-        <is>
-          <t>Nipel motorlu kaldırma sistemi (0,75 kW çift redüktörlü frenli kaldırma motoru, mafsal 50'lik boru, UCP bilya, kontrol panosu dâhil)</t>
-        </is>
-      </c>
-      <c r="D11" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E11" s="20" t="n">
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>HZC-SLO-004</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Yem silosu ve nakil sistemi — En az 17,77 ton galvaniz kaplama sac silo, helezonlu merdiven, 0,75 kW yem nakil motoru, 22 m PVC nakil hattı</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>50000</v>
+        <v>172996.93</v>
       </c>
       <c r="G11" s="5">
         <f>ROUND(E11*F11,2)</f>
@@ -4538,282 +4538,42 @@
         </is>
       </c>
       <c r="B12" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="C12" s="16" t="inlineStr">
-        <is>
-          <t>140 x 140 cm tünel havalandırma fanı</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E12" s="20" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>Montaj ve nakliye — Kümes montajı ve nakliye bedelleri</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>2</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>25500</v>
+        <v>225000</v>
       </c>
       <c r="G12" s="5">
         <f>ROUND(E12*F12,2)</f>
         <v/>
       </c>
     </row>
-    <row r="13" ht="14" customHeight="1">
-      <c r="A13" s="17" t="inlineStr">
-        <is>
-          <t>Makine ve ekipman alımı</t>
-        </is>
-      </c>
-      <c r="B13" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="C13" s="16" t="inlineStr">
-        <is>
-          <t>3 makaralı klape (hava giriş kapağı)</t>
-        </is>
-      </c>
-      <c r="D13" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E13" s="20" t="n">
-        <v>60</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>1200</v>
-      </c>
-      <c r="G13" s="5">
-        <f>ROUND(E13*F13,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="14" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
-        <is>
-          <t>Makine ve ekipman alımı</t>
-        </is>
-      </c>
-      <c r="B14" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="C14" s="16" t="inlineStr">
-        <is>
-          <t>Klape açma sistemi</t>
-        </is>
-      </c>
-      <c r="D14" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E14" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>11000</v>
-      </c>
-      <c r="G14" s="5">
-        <f>ROUND(E14*F14,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
-        <is>
-          <t>Makine ve ekipman alımı</t>
-        </is>
-      </c>
-      <c r="B15" s="19" t="n">
-        <v>11</v>
-      </c>
-      <c r="C15" s="16" t="inlineStr">
-        <is>
-          <t>7 inç dokunmatik ekran kümes kontrol panosu (uzaktan erişim, karbondioksit, nem ve basınç sensörü, 5 ısı sensörü dâhil)</t>
-        </is>
-      </c>
-      <c r="D15" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E15" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>210000</v>
-      </c>
-      <c r="G15" s="5">
-        <f>ROUND(E15*F15,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>Makine ve ekipman alımı</t>
-        </is>
-      </c>
-      <c r="B16" s="19" t="n">
-        <v>12</v>
-      </c>
-      <c r="C16" s="16" t="inlineStr">
-        <is>
-          <t>15 m x 1,5 m x 15 cm PVC çerçeveli, kendinden depolu ve su pompalı tüp ped (serinletme) sistemi</t>
-        </is>
-      </c>
-      <c r="D16" s="19" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E16" s="20" t="n">
-        <v>45.72</v>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>4500</v>
-      </c>
-      <c r="G16" s="5">
-        <f>ROUND(E16*F16,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="14" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>Makine ve ekipman alımı</t>
-        </is>
-      </c>
-      <c r="B17" s="19" t="n">
-        <v>13</v>
-      </c>
-      <c r="C17" s="16" t="inlineStr">
-        <is>
-          <t>Ped kapağı açma sistemi</t>
-        </is>
-      </c>
-      <c r="D17" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E17" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>11000</v>
-      </c>
-      <c r="G17" s="5">
-        <f>ROUND(E17*F17,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="14" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>Makine ve ekipman alımı</t>
-        </is>
-      </c>
-      <c r="B18" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="C18" s="16" t="inlineStr">
-        <is>
-          <t>110 x 150 cm ped kapağı</t>
-        </is>
-      </c>
-      <c r="D18" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E18" s="20" t="n">
-        <v>40</v>
-      </c>
-      <c r="F18" s="5" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G18" s="5">
-        <f>ROUND(E18*F18,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="14" customHeight="1">
-      <c r="A19" s="17" t="inlineStr">
-        <is>
-          <t>Makine ve ekipman alımı</t>
-        </is>
-      </c>
-      <c r="B19" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="C19" s="16" t="inlineStr">
-        <is>
-          <t>18 ton galvaniz yem silosu ve alt grubu</t>
-        </is>
-      </c>
-      <c r="D19" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E19" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>155000</v>
-      </c>
-      <c r="G19" s="5">
-        <f>ROUND(E19*F19,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="14" customHeight="1">
-      <c r="A20" s="17" t="inlineStr">
-        <is>
-          <t>Makine ve ekipman alımı</t>
-        </is>
-      </c>
-      <c r="B20" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="C20" s="16" t="inlineStr">
-        <is>
-          <t>İşçilik ve nakliye</t>
-        </is>
-      </c>
-      <c r="D20" s="19" t="inlineStr">
-        <is>
-          <t>tk</t>
-        </is>
-      </c>
-      <c r="E20" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="F20" s="5" t="n">
-        <v>250000</v>
-      </c>
-      <c r="G20" s="5">
-        <f>ROUND(E20*F20,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="21" t="n"/>
-      <c r="B21" s="21" t="n"/>
-      <c r="C21" s="22" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="21" t="n"/>
+      <c r="B13" s="21" t="n"/>
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>MAKİNE-EKİPMAN TOPLAMI (KDV hariç)</t>
         </is>
       </c>
-      <c r="D21" s="21" t="n"/>
-      <c r="E21" s="21" t="n"/>
-      <c r="F21" s="21" t="n"/>
-      <c r="G21" s="9">
-        <f>SUM(G5:G20)</f>
+      <c r="D13" s="21" t="n"/>
+      <c r="E13" s="21" t="n"/>
+      <c r="F13" s="21" t="n"/>
+      <c r="G13" s="9">
+        <f>SUM(G5:G12)</f>
         <v/>
       </c>
     </row>
@@ -7174,7 +6934,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>24974467.25</v>
+        <v>24988354.46</v>
       </c>
       <c r="C5" s="6">
         <f>B5/52.7585</f>
@@ -7231,7 +6991,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>2871960</v>
+        <v>2885847.21</v>
       </c>
       <c r="C8" s="6">
         <f>B8/52.7585</f>
@@ -7269,7 +7029,7 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>9200012.75</v>
+        <v>9213899.960000001</v>
       </c>
       <c r="C10" s="10">
         <f>B10/52.7585</f>
@@ -7307,7 +7067,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>4994893.45</v>
+        <v>4997670.89</v>
       </c>
       <c r="C12" s="6">
         <f>B12/52.7585</f>

</xml_diff>

<commit_message>
Yayin: kapasite 36.000, sihhi tesisat proformada, is plani Word nushasi
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
+++ b/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
@@ -4471,7 +4471,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Makine ve ekipman alımı</t>
@@ -4487,7 +4487,7 @@
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>Klape sistemi — 40 adet 26 x 56 cm izolasyonlu plastik klape, klape başına 1.750 m³/h, 2 aktüatörlü açma-kapama, 161 m hat</t>
+          <t>Klape sistemi — 30 adet 26 x 56 cm izolasyonlu plastik klape, klape başına 1.750 m³/h (30 x 1.750 = 52.500 m³/h, mekanik projedeki 46.717 m³/h ihtiyacının üzerinde), 2 aktüatörlü açma-kapama, 161 m hat</t>
         </is>
       </c>
       <c r="E10" s="19" t="n">

</xml_diff>

<commit_message>
Yayin: sihhi tesisat kalemleri fiyatlandirildi
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
+++ b/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>'A3.4-EK Yapım'!H56</f>
+        <f>'A3.4-EK Yapım'!H72</f>
         <v/>
       </c>
       <c r="C12" s="6">
@@ -4591,7 +4591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4614,7 +4614,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Kümes A ve B blokları dışındaki yapılar ile bu iki bloktan hibe kapsamı dışına çıkarılan pozlar. Bu imalatlar yapılmaya devam eder; teklif alma usulüne tabi değildir, proforma fatura ile beyan edilir ve tamamı öz kaynaktan karşılanır. Birim fiyatlar, hibe kapsamındaki işlerle aynı esasa göre kurulmuştur: ÇŞB 2026 ve TKDK 17.02.2026 kitap fiyatlarına %16 tenzilat uygulanmıştır.</t>
+          <t>Kümes A ve B blokları dışındaki yapılar ile bu iki bloktan hibe kapsamı dışına çıkarılan pozlar. Bu imalatlar yapılmaya devam eder; teklif alma usulüne tabi değildir, proforma fatura ile beyan edilir ve tamamı öz kaynaktan karşılanır. Birim fiyatlar, hibe kapsamındaki işlerle aynı esasa göre kurulmuştur: ÇŞB 2026 ve TKDK 17.02.2026 kitap fiyatlarına %16 tenzilat uygulanmıştır. Sayfanın sonundaki SIHHİ TESİSAT bölümü keşif özetinde yer almaz: miktarları onaylı sıhhi tesisat projesinden, birim fiyatları piyasa araştırmasından gelir; kitap fiyatı olmadığı için o kalemlere tenzilat uygulanmaz. Bu sayfa 36 numaralı proforma ile kuruşu kuruşuna aynıdır.</t>
         </is>
       </c>
     </row>
@@ -6548,25 +6548,588 @@
         <v/>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="21" t="n"/>
-      <c r="B56" s="21" t="n"/>
-      <c r="C56" s="21" t="n"/>
-      <c r="D56" s="22" t="inlineStr">
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>SIHHİ TESİSAT — keşif özetinde yer almaz; miktarlar onaylı sıhhi tesisat projesinden, birim fiyatlar piyasa araştırmasından (kitap fiyatı olmadığı için %16 tenzilat uygulanmaz)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="17" t="inlineStr">
+        <is>
+          <t>Sıhhi tesisat</t>
+        </is>
+      </c>
+      <c r="B57" s="17" t="inlineStr">
+        <is>
+          <t>Kümes A Blok</t>
+        </is>
+      </c>
+      <c r="C57" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>Temiz su tesisatı — PPRC boru ve ek parçaları, 1/2" - 1 1/4" kolon ve kat tesisatı, küresel vanalar, boru askı ve kılıfları (kolon şemasına göre)</t>
+        </is>
+      </c>
+      <c r="E57" s="19" t="inlineStr">
+        <is>
+          <t>tk</t>
+        </is>
+      </c>
+      <c r="F57" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="5" t="n">
+        <v>38000</v>
+      </c>
+      <c r="H57" s="5">
+        <f>ROUND(F57*G57,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="17" t="inlineStr">
+        <is>
+          <t>Sıhhi tesisat</t>
+        </is>
+      </c>
+      <c r="B58" s="17" t="inlineStr">
+        <is>
+          <t>Kümes A Blok</t>
+        </is>
+      </c>
+      <c r="C58" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D58" s="16" t="inlineStr">
+        <is>
+          <t>Pis su tesisatı — Ø50 / Ø70 / Ø100 sert PVC boru, kolon ve yatay hatlar, temizleme kapakları, yer süzgeçleri</t>
+        </is>
+      </c>
+      <c r="E58" s="19" t="inlineStr">
+        <is>
+          <t>tk</t>
+        </is>
+      </c>
+      <c r="F58" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" s="5" t="n">
+        <v>27000</v>
+      </c>
+      <c r="H58" s="5">
+        <f>ROUND(F58*G58,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>Sıhhi tesisat</t>
+        </is>
+      </c>
+      <c r="B59" s="17" t="inlineStr">
+        <is>
+          <t>Kümes A Blok</t>
+        </is>
+      </c>
+      <c r="C59" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>Vitrifiye ve armatür grubu — lavabo, klozet, alaturka hela taşı, duş teknesi, evye, pisuvar ve bataryaları (servis bölümü)</t>
+        </is>
+      </c>
+      <c r="E59" s="19" t="inlineStr">
+        <is>
+          <t>tk</t>
+        </is>
+      </c>
+      <c r="F59" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="5" t="n">
+        <v>42000</v>
+      </c>
+      <c r="H59" s="5">
+        <f>ROUND(F59*G59,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t>Sıhhi tesisat</t>
+        </is>
+      </c>
+      <c r="B60" s="17" t="inlineStr">
+        <is>
+          <t>Kümes A Blok</t>
+        </is>
+      </c>
+      <c r="C60" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D60" s="16" t="inlineStr">
+        <is>
+          <t>Termosifon — sıcak su üretimi (proje raporu: sıcak su hatları termosifon vasıtasıyla)</t>
+        </is>
+      </c>
+      <c r="E60" s="19" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="F60" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="5" t="n">
+        <v>13000</v>
+      </c>
+      <c r="H60" s="5">
+        <f>ROUND(F60*G60,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" ht="30" customHeight="1">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>Sıhhi tesisat</t>
+        </is>
+      </c>
+      <c r="B61" s="17" t="inlineStr">
+        <is>
+          <t>Kümes B Blok</t>
+        </is>
+      </c>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>Temiz su tesisatı — PPRC boru ve ek parçaları, 1/2" - 1 1/4" kolon ve kat tesisatı, küresel vanalar, boru askı ve kılıfları (kolon şemasına göre)</t>
+        </is>
+      </c>
+      <c r="E61" s="19" t="inlineStr">
+        <is>
+          <t>tk</t>
+        </is>
+      </c>
+      <c r="F61" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="5" t="n">
+        <v>38000</v>
+      </c>
+      <c r="H61" s="5">
+        <f>ROUND(F61*G61,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="17" t="inlineStr">
+        <is>
+          <t>Sıhhi tesisat</t>
+        </is>
+      </c>
+      <c r="B62" s="17" t="inlineStr">
+        <is>
+          <t>Kümes B Blok</t>
+        </is>
+      </c>
+      <c r="C62" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>Pis su tesisatı — Ø50 / Ø70 / Ø100 sert PVC boru, kolon ve yatay hatlar, temizleme kapakları, yer süzgeçleri</t>
+        </is>
+      </c>
+      <c r="E62" s="19" t="inlineStr">
+        <is>
+          <t>tk</t>
+        </is>
+      </c>
+      <c r="F62" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" s="5" t="n">
+        <v>27000</v>
+      </c>
+      <c r="H62" s="5">
+        <f>ROUND(F62*G62,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t>Sıhhi tesisat</t>
+        </is>
+      </c>
+      <c r="B63" s="17" t="inlineStr">
+        <is>
+          <t>Kümes B Blok</t>
+        </is>
+      </c>
+      <c r="C63" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>Vitrifiye ve armatür grubu — lavabo, klozet, alaturka hela taşı, duş teknesi, evye, pisuvar ve bataryaları (servis bölümü)</t>
+        </is>
+      </c>
+      <c r="E63" s="19" t="inlineStr">
+        <is>
+          <t>tk</t>
+        </is>
+      </c>
+      <c r="F63" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" s="5" t="n">
+        <v>42000</v>
+      </c>
+      <c r="H63" s="5">
+        <f>ROUND(F63*G63,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="17" t="inlineStr">
+        <is>
+          <t>Sıhhi tesisat</t>
+        </is>
+      </c>
+      <c r="B64" s="17" t="inlineStr">
+        <is>
+          <t>Kümes B Blok</t>
+        </is>
+      </c>
+      <c r="C64" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>Termosifon — sıcak su üretimi (proje raporu: sıcak su hatları termosifon vasıtasıyla)</t>
+        </is>
+      </c>
+      <c r="E64" s="19" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="F64" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="5" t="n">
+        <v>13000</v>
+      </c>
+      <c r="H64" s="5">
+        <f>ROUND(F64*G64,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="14" customHeight="1">
+      <c r="A65" s="17" t="inlineStr">
+        <is>
+          <t>Sıhhi tesisat</t>
+        </is>
+      </c>
+      <c r="B65" s="17" t="inlineStr">
+        <is>
+          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
+        </is>
+      </c>
+      <c r="C65" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>Şebeke su bağlantısı ve 2" su sayacı — temiz su girişi 80 YB</t>
+        </is>
+      </c>
+      <c r="E65" s="19" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="F65" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" s="5" t="n">
+        <v>26000</v>
+      </c>
+      <c r="H65" s="5">
+        <f>ROUND(F65*G65,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" ht="14" customHeight="1">
+      <c r="A66" s="17" t="inlineStr">
+        <is>
+          <t>Sıhhi tesisat</t>
+        </is>
+      </c>
+      <c r="B66" s="17" t="inlineStr">
+        <is>
+          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
+        </is>
+      </c>
+      <c r="C66" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D66" s="16" t="inlineStr">
+        <is>
+          <t>Hidrofor — Q = 2 m³/h, P = 33-38 mSS</t>
+        </is>
+      </c>
+      <c r="E66" s="19" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="F66" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" s="5" t="n">
+        <v>48000</v>
+      </c>
+      <c r="H66" s="5">
+        <f>ROUND(F66*G66,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67" ht="14" customHeight="1">
+      <c r="A67" s="17" t="inlineStr">
+        <is>
+          <t>Sıhhi tesisat</t>
+        </is>
+      </c>
+      <c r="B67" s="17" t="inlineStr">
+        <is>
+          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
+        </is>
+      </c>
+      <c r="C67" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D67" s="16" t="inlineStr">
+        <is>
+          <t>Tesisat hidroforu — 0,3 m³/h, 30 mSS (3A)</t>
+        </is>
+      </c>
+      <c r="E67" s="19" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="F67" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" s="5" t="n">
+        <v>19000</v>
+      </c>
+      <c r="H67" s="5">
+        <f>ROUND(F67*G67,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68" ht="14" customHeight="1">
+      <c r="A68" s="17" t="inlineStr">
+        <is>
+          <t>Sıhhi tesisat</t>
+        </is>
+      </c>
+      <c r="B68" s="17" t="inlineStr">
+        <is>
+          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
+        </is>
+      </c>
+      <c r="C68" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>Modüler galvaniz su deposu — 3 ton (3A)</t>
+        </is>
+      </c>
+      <c r="E68" s="19" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="F68" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" s="5" t="n">
+        <v>36000</v>
+      </c>
+      <c r="H68" s="5">
+        <f>ROUND(F68*G68,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="17" t="inlineStr">
+        <is>
+          <t>Sıhhi tesisat</t>
+        </is>
+      </c>
+      <c r="B69" s="17" t="inlineStr">
+        <is>
+          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
+        </is>
+      </c>
+      <c r="C69" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D69" s="16" t="inlineStr">
+        <is>
+          <t>Yağmur suyu geri kazanım deposu — modüler galvaniz 10 ton, 1,08 x 1,08 x 2,66 m</t>
+        </is>
+      </c>
+      <c r="E69" s="19" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="F69" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" s="5" t="n">
+        <v>88000</v>
+      </c>
+      <c r="H69" s="5">
+        <f>ROUND(F69*G69,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="30" customHeight="1">
+      <c r="A70" s="17" t="inlineStr">
+        <is>
+          <t>Sıhhi tesisat</t>
+        </is>
+      </c>
+      <c r="B70" s="17" t="inlineStr">
+        <is>
+          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
+        </is>
+      </c>
+      <c r="C70" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D70" s="16" t="inlineStr">
+        <is>
+          <t>Yağmur suyu geri kazanım donanımı — pislik tutucu ve emiş filtresi, akış yavaşlatıcı, taşkan sifonu (4 m³/h), tam otomatik kum filtresi DN160, su sayacı ve otomatik kontrol</t>
+        </is>
+      </c>
+      <c r="E70" s="19" t="inlineStr">
+        <is>
+          <t>tk</t>
+        </is>
+      </c>
+      <c r="F70" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="5" t="n">
+        <v>125000</v>
+      </c>
+      <c r="H70" s="5">
+        <f>ROUND(F70*G70,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="14" customHeight="1">
+      <c r="A71" s="17" t="inlineStr">
+        <is>
+          <t>Sıhhi tesisat</t>
+        </is>
+      </c>
+      <c r="B71" s="17" t="inlineStr">
+        <is>
+          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
+        </is>
+      </c>
+      <c r="C71" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D71" s="16" t="inlineStr">
+        <is>
+          <t>Bahçe sulama pompası — 0,5 m³/h, 40 mSS, 0,5 kW</t>
+        </is>
+      </c>
+      <c r="E71" s="19" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="F71" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" s="5" t="n">
+        <v>16000</v>
+      </c>
+      <c r="H71" s="5">
+        <f>ROUND(F71*G71,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="21" t="n"/>
+      <c r="B72" s="21" t="n"/>
+      <c r="C72" s="21" t="n"/>
+      <c r="D72" s="22" t="inlineStr">
         <is>
           <t>HİBE DIŞI YAPIM İŞLERİ TOPLAMI (KDV hariç)</t>
         </is>
       </c>
-      <c r="E56" s="21" t="n"/>
-      <c r="F56" s="21" t="n"/>
-      <c r="G56" s="21" t="n"/>
-      <c r="H56" s="9">
-        <f>SUM(H5:H55)</f>
+      <c r="E72" s="21" t="n"/>
+      <c r="F72" s="21" t="n"/>
+      <c r="G72" s="21" t="n"/>
+      <c r="H72" s="9">
+        <f>SUM(H5:H71)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A56:H56"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6934,7 +7497,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>24988354.46</v>
+        <v>25586354.46</v>
       </c>
       <c r="C5" s="6">
         <f>B5/52.7585</f>
@@ -6972,7 +7535,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>5618052.75</v>
+        <v>6216052.75</v>
       </c>
       <c r="C7" s="6">
         <f>B7/52.7585</f>
@@ -7029,7 +7592,7 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>9213899.960000001</v>
+        <v>9811899.960000001</v>
       </c>
       <c r="C10" s="10">
         <f>B10/52.7585</f>
@@ -7067,7 +7630,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>4997670.89</v>
+        <v>5117270.89</v>
       </c>
       <c r="C12" s="6">
         <f>B12/52.7585</f>

</xml_diff>

<commit_message>
Yayin: sihhi tesisattan bes kalem cikarildi
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
+++ b/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>'A3.4-EK Yapım'!H72</f>
+        <f>'A3.4-EK Yapım'!H66</f>
         <v/>
       </c>
       <c r="C12" s="6">
@@ -4591,7 +4591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -6647,26 +6647,26 @@
       </c>
       <c r="D59" s="16" t="inlineStr">
         <is>
-          <t>Vitrifiye ve armatür grubu — lavabo, klozet, alaturka hela taşı, duş teknesi, evye, pisuvar ve bataryaları (servis bölümü)</t>
+          <t>Termosifon — sıcak su üretimi (proje raporu: sıcak su hatları termosifon vasıtasıyla)</t>
         </is>
       </c>
       <c r="E59" s="19" t="inlineStr">
         <is>
-          <t>tk</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="F59" s="20" t="n">
         <v>1</v>
       </c>
       <c r="G59" s="5" t="n">
-        <v>42000</v>
+        <v>13000</v>
       </c>
       <c r="H59" s="5">
         <f>ROUND(F59*G59,2)</f>
         <v/>
       </c>
     </row>
-    <row r="60" ht="20" customHeight="1">
+    <row r="60" ht="30" customHeight="1">
       <c r="A60" s="17" t="inlineStr">
         <is>
           <t>Sıhhi tesisat</t>
@@ -6674,7 +6674,7 @@
       </c>
       <c r="B60" s="17" t="inlineStr">
         <is>
-          <t>Kümes A Blok</t>
+          <t>Kümes B Blok</t>
         </is>
       </c>
       <c r="C60" s="19" t="inlineStr">
@@ -6684,26 +6684,26 @@
       </c>
       <c r="D60" s="16" t="inlineStr">
         <is>
-          <t>Termosifon — sıcak su üretimi (proje raporu: sıcak su hatları termosifon vasıtasıyla)</t>
+          <t>Temiz su tesisatı — PPRC boru ve ek parçaları, 1/2" - 1 1/4" kolon ve kat tesisatı, küresel vanalar, boru askı ve kılıfları (kolon şemasına göre)</t>
         </is>
       </c>
       <c r="E60" s="19" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>tk</t>
         </is>
       </c>
       <c r="F60" s="20" t="n">
         <v>1</v>
       </c>
       <c r="G60" s="5" t="n">
-        <v>13000</v>
+        <v>38000</v>
       </c>
       <c r="H60" s="5">
         <f>ROUND(F60*G60,2)</f>
         <v/>
       </c>
     </row>
-    <row r="61" ht="30" customHeight="1">
+    <row r="61" ht="20" customHeight="1">
       <c r="A61" s="17" t="inlineStr">
         <is>
           <t>Sıhhi tesisat</t>
@@ -6721,7 +6721,7 @@
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>Temiz su tesisatı — PPRC boru ve ek parçaları, 1/2" - 1 1/4" kolon ve kat tesisatı, küresel vanalar, boru askı ve kılıfları (kolon şemasına göre)</t>
+          <t>Pis su tesisatı — Ø50 / Ø70 / Ø100 sert PVC boru, kolon ve yatay hatlar, temizleme kapakları, yer süzgeçleri</t>
         </is>
       </c>
       <c r="E61" s="19" t="inlineStr">
@@ -6733,7 +6733,7 @@
         <v>1</v>
       </c>
       <c r="G61" s="5" t="n">
-        <v>38000</v>
+        <v>27000</v>
       </c>
       <c r="H61" s="5">
         <f>ROUND(F61*G61,2)</f>
@@ -6758,26 +6758,26 @@
       </c>
       <c r="D62" s="16" t="inlineStr">
         <is>
-          <t>Pis su tesisatı — Ø50 / Ø70 / Ø100 sert PVC boru, kolon ve yatay hatlar, temizleme kapakları, yer süzgeçleri</t>
+          <t>Termosifon — sıcak su üretimi (proje raporu: sıcak su hatları termosifon vasıtasıyla)</t>
         </is>
       </c>
       <c r="E62" s="19" t="inlineStr">
         <is>
-          <t>tk</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="F62" s="20" t="n">
         <v>1</v>
       </c>
       <c r="G62" s="5" t="n">
-        <v>27000</v>
+        <v>13000</v>
       </c>
       <c r="H62" s="5">
         <f>ROUND(F62*G62,2)</f>
         <v/>
       </c>
     </row>
-    <row r="63" ht="20" customHeight="1">
+    <row r="63" ht="14" customHeight="1">
       <c r="A63" s="17" t="inlineStr">
         <is>
           <t>Sıhhi tesisat</t>
@@ -6785,7 +6785,7 @@
       </c>
       <c r="B63" s="17" t="inlineStr">
         <is>
-          <t>Kümes B Blok</t>
+          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
         </is>
       </c>
       <c r="C63" s="19" t="inlineStr">
@@ -6795,26 +6795,26 @@
       </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
-          <t>Vitrifiye ve armatür grubu — lavabo, klozet, alaturka hela taşı, duş teknesi, evye, pisuvar ve bataryaları (servis bölümü)</t>
+          <t>Şebeke su bağlantısı ve 2" su sayacı — temiz su girişi 80 YB</t>
         </is>
       </c>
       <c r="E63" s="19" t="inlineStr">
         <is>
-          <t>tk</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="F63" s="20" t="n">
         <v>1</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>42000</v>
+        <v>26000</v>
       </c>
       <c r="H63" s="5">
         <f>ROUND(F63*G63,2)</f>
         <v/>
       </c>
     </row>
-    <row r="64" ht="20" customHeight="1">
+    <row r="64" ht="14" customHeight="1">
       <c r="A64" s="17" t="inlineStr">
         <is>
           <t>Sıhhi tesisat</t>
@@ -6822,7 +6822,7 @@
       </c>
       <c r="B64" s="17" t="inlineStr">
         <is>
-          <t>Kümes B Blok</t>
+          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
         </is>
       </c>
       <c r="C64" s="19" t="inlineStr">
@@ -6832,7 +6832,7 @@
       </c>
       <c r="D64" s="16" t="inlineStr">
         <is>
-          <t>Termosifon — sıcak su üretimi (proje raporu: sıcak su hatları termosifon vasıtasıyla)</t>
+          <t>Hidrofor — Q = 2 m³/h, P = 33-38 mSS</t>
         </is>
       </c>
       <c r="E64" s="19" t="inlineStr">
@@ -6844,7 +6844,7 @@
         <v>1</v>
       </c>
       <c r="G64" s="5" t="n">
-        <v>13000</v>
+        <v>48000</v>
       </c>
       <c r="H64" s="5">
         <f>ROUND(F64*G64,2)</f>
@@ -6869,7 +6869,7 @@
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>Şebeke su bağlantısı ve 2" su sayacı — temiz su girişi 80 YB</t>
+          <t>Tesisat hidroforu — 0,3 m³/h, 30 mSS (3A)</t>
         </is>
       </c>
       <c r="E65" s="19" t="inlineStr">
@@ -6881,249 +6881,27 @@
         <v>1</v>
       </c>
       <c r="G65" s="5" t="n">
-        <v>26000</v>
+        <v>19000</v>
       </c>
       <c r="H65" s="5">
         <f>ROUND(F65*G65,2)</f>
         <v/>
       </c>
     </row>
-    <row r="66" ht="14" customHeight="1">
-      <c r="A66" s="17" t="inlineStr">
-        <is>
-          <t>Sıhhi tesisat</t>
-        </is>
-      </c>
-      <c r="B66" s="17" t="inlineStr">
-        <is>
-          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
-        </is>
-      </c>
-      <c r="C66" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D66" s="16" t="inlineStr">
-        <is>
-          <t>Hidrofor — Q = 2 m³/h, P = 33-38 mSS</t>
-        </is>
-      </c>
-      <c r="E66" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="F66" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G66" s="5" t="n">
-        <v>48000</v>
-      </c>
-      <c r="H66" s="5">
-        <f>ROUND(F66*G66,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67" ht="14" customHeight="1">
-      <c r="A67" s="17" t="inlineStr">
-        <is>
-          <t>Sıhhi tesisat</t>
-        </is>
-      </c>
-      <c r="B67" s="17" t="inlineStr">
-        <is>
-          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
-        </is>
-      </c>
-      <c r="C67" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D67" s="16" t="inlineStr">
-        <is>
-          <t>Tesisat hidroforu — 0,3 m³/h, 30 mSS (3A)</t>
-        </is>
-      </c>
-      <c r="E67" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="F67" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G67" s="5" t="n">
-        <v>19000</v>
-      </c>
-      <c r="H67" s="5">
-        <f>ROUND(F67*G67,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68" ht="14" customHeight="1">
-      <c r="A68" s="17" t="inlineStr">
-        <is>
-          <t>Sıhhi tesisat</t>
-        </is>
-      </c>
-      <c r="B68" s="17" t="inlineStr">
-        <is>
-          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
-        </is>
-      </c>
-      <c r="C68" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D68" s="16" t="inlineStr">
-        <is>
-          <t>Modüler galvaniz su deposu — 3 ton (3A)</t>
-        </is>
-      </c>
-      <c r="E68" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="F68" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G68" s="5" t="n">
-        <v>36000</v>
-      </c>
-      <c r="H68" s="5">
-        <f>ROUND(F68*G68,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69" ht="20" customHeight="1">
-      <c r="A69" s="17" t="inlineStr">
-        <is>
-          <t>Sıhhi tesisat</t>
-        </is>
-      </c>
-      <c r="B69" s="17" t="inlineStr">
-        <is>
-          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
-        </is>
-      </c>
-      <c r="C69" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D69" s="16" t="inlineStr">
-        <is>
-          <t>Yağmur suyu geri kazanım deposu — modüler galvaniz 10 ton, 1,08 x 1,08 x 2,66 m</t>
-        </is>
-      </c>
-      <c r="E69" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="F69" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G69" s="5" t="n">
-        <v>88000</v>
-      </c>
-      <c r="H69" s="5">
-        <f>ROUND(F69*G69,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70" ht="30" customHeight="1">
-      <c r="A70" s="17" t="inlineStr">
-        <is>
-          <t>Sıhhi tesisat</t>
-        </is>
-      </c>
-      <c r="B70" s="17" t="inlineStr">
-        <is>
-          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
-        </is>
-      </c>
-      <c r="C70" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D70" s="16" t="inlineStr">
-        <is>
-          <t>Yağmur suyu geri kazanım donanımı — pislik tutucu ve emiş filtresi, akış yavaşlatıcı, taşkan sifonu (4 m³/h), tam otomatik kum filtresi DN160, su sayacı ve otomatik kontrol</t>
-        </is>
-      </c>
-      <c r="E70" s="19" t="inlineStr">
-        <is>
-          <t>tk</t>
-        </is>
-      </c>
-      <c r="F70" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G70" s="5" t="n">
-        <v>125000</v>
-      </c>
-      <c r="H70" s="5">
-        <f>ROUND(F70*G70,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71" ht="14" customHeight="1">
-      <c r="A71" s="17" t="inlineStr">
-        <is>
-          <t>Sıhhi tesisat</t>
-        </is>
-      </c>
-      <c r="B71" s="17" t="inlineStr">
-        <is>
-          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
-        </is>
-      </c>
-      <c r="C71" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D71" s="16" t="inlineStr">
-        <is>
-          <t>Bahçe sulama pompası — 0,5 m³/h, 40 mSS, 0,5 kW</t>
-        </is>
-      </c>
-      <c r="E71" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="F71" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G71" s="5" t="n">
-        <v>16000</v>
-      </c>
-      <c r="H71" s="5">
-        <f>ROUND(F71*G71,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="21" t="n"/>
-      <c r="B72" s="21" t="n"/>
-      <c r="C72" s="21" t="n"/>
-      <c r="D72" s="22" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="21" t="n"/>
+      <c r="B66" s="21" t="n"/>
+      <c r="C66" s="21" t="n"/>
+      <c r="D66" s="22" t="inlineStr">
         <is>
           <t>HİBE DIŞI YAPIM İŞLERİ TOPLAMI (KDV hariç)</t>
         </is>
       </c>
-      <c r="E72" s="21" t="n"/>
-      <c r="F72" s="21" t="n"/>
-      <c r="G72" s="21" t="n"/>
-      <c r="H72" s="9">
-        <f>SUM(H5:H71)</f>
+      <c r="E66" s="21" t="n"/>
+      <c r="F66" s="21" t="n"/>
+      <c r="G66" s="21" t="n"/>
+      <c r="H66" s="9">
+        <f>SUM(H5:H65)</f>
         <v/>
       </c>
     </row>
@@ -7497,7 +7275,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>25586354.46</v>
+        <v>25237354.46</v>
       </c>
       <c r="C5" s="6">
         <f>B5/52.7585</f>
@@ -7535,7 +7313,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>6216052.75</v>
+        <v>5867052.75</v>
       </c>
       <c r="C7" s="6">
         <f>B7/52.7585</f>
@@ -7592,7 +7370,7 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>9811899.960000001</v>
+        <v>9462899.960000001</v>
       </c>
       <c r="C10" s="10">
         <f>B10/52.7585</f>
@@ -7630,7 +7408,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>5117270.89</v>
+        <v>5047470.89</v>
       </c>
       <c r="C12" s="6">
         <f>B12/52.7585</f>

</xml_diff>

<commit_message>
Yayın: foseptik bedeli önceki inşaat proformasına sabitlendi
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
+++ b/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
@@ -5912,7 +5912,7 @@
         <v>1</v>
       </c>
       <c r="G42" s="5" t="n">
-        <v>55000</v>
+        <v>76961.66</v>
       </c>
       <c r="H42" s="5">
         <f>ROUND(F42*G42,2)</f>
@@ -7053,7 +7053,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>25161130.8</v>
+        <v>25183092.46</v>
       </c>
       <c r="C5" s="6">
         <f>B5/52.7585</f>
@@ -7091,7 +7091,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>5845091.09</v>
+        <v>5867052.75</v>
       </c>
       <c r="C7" s="6">
         <f>B7/52.7585</f>
@@ -7148,7 +7148,7 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>9440938.300000001</v>
+        <v>9462899.960000001</v>
       </c>
       <c r="C10" s="10">
         <f>B10/52.7585</f>
@@ -7186,7 +7186,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>5032226.16</v>
+        <v>5036618.49</v>
       </c>
       <c r="C12" s="6">
         <f>B12/52.7585</f>

</xml_diff>

<commit_message>
Yayın: makine-ekipman gideri tek proformaya bağlandı, ısıtma lotu iptal
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
+++ b/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>'A3.4-EK Makine-Ekipman'!G13</f>
+        <f>'A3.4-EK Makine-Ekipman'!G15</f>
         <v/>
       </c>
       <c r="C13" s="6">
@@ -736,59 +736,40 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Hibe dışı kümes ısıtma sistemi</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="n">
-        <v>710000</v>
-      </c>
-      <c r="C14" s="6">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>UYGUN OLMAYAN HARCAMA (öz kaynak)</t>
+        </is>
+      </c>
+      <c r="B14" s="9">
+        <f>B12+B13</f>
+        <v/>
+      </c>
+      <c r="C14" s="10">
         <f>B14/52.7585</f>
         <v/>
       </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>Ayrı lot; proforma ile beyan</t>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Tamamı öz kaynaktan karşılanır</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>UYGUN OLMAYAN HARCAMA (öz kaynak)</t>
-        </is>
-      </c>
-      <c r="B15" s="9">
-        <f>B12+B13+B14</f>
-        <v/>
-      </c>
-      <c r="C15" s="10">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>TOPLAM YATIRIM (KDV hariç)</t>
+        </is>
+      </c>
+      <c r="B15" s="13">
+        <f>B9+B14</f>
+        <v/>
+      </c>
+      <c r="C15" s="14">
         <f>B15/52.7585</f>
         <v/>
       </c>
-      <c r="D15" s="11" t="inlineStr">
-        <is>
-          <t>Tamamı öz kaynaktan karşılanır</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>TOPLAM YATIRIM (KDV hariç)</t>
-        </is>
-      </c>
-      <c r="B16" s="13">
-        <f>B9+B15</f>
-        <v/>
-      </c>
-      <c r="C16" s="14">
-        <f>B16/52.7585</f>
-        <v/>
-      </c>
-      <c r="D16" s="15" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>Uygun harcama + uygun olmayan harcama</t>
         </is>
@@ -4109,7 +4090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4189,14 +4170,14 @@
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>Yemleme sistemi — 3 hat, 243 m hat uzunluğu, 150 kg galvanizli yem deposu x 3, 0,55 kW yemlik motoru x 3, 35 cm çapında 324 plastik yemlik, 1,1 kW çift redüktörlü frenli otomatik kaldırma</t>
+          <t>Otomatik spiral yemlik sistemi (depo motor grubu ve kaldırma dâhil) — 3 hat, 243 m yemlik hattı, 150 kg galvanizli yem deposu x 3, 0,55 kW yemlik motoru x 3, 35 cm çapında 324 plastik yemlik, 1,1 kW çift redüktörlü frenli otomatik kaldırma</t>
         </is>
       </c>
       <c r="E5" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>250062.04</v>
+        <v>251748</v>
       </c>
       <c r="G5" s="5">
         <f>ROUND(E5*F5,2)</f>
@@ -4214,26 +4195,26 @@
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>HZC-COM-004</t>
+          <t>HZC-WTR-005</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>Kümes kontrol panosu — HZC-70 işlemcili; 5 sıcaklık, 1 nem, 1 basınç ve 1 CO2 sensörü, alarm sistemi, uzaktan erişim, PLC kontrol, raporlama ve analiz</t>
+          <t>Otomatik nipel suluk sistemi (regülatör, hat sonu ve kaldırma dâhil) — Kümes başına 4 hat, toplam 312 m hat, 22 x 22 mm hat çapı, 1.560 metal 360° nipel suluk, 4 regülatör, 4 hat sonu, 0,75 kW çift redüktörlü frenli otomatik kaldırma</t>
         </is>
       </c>
       <c r="E6" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>262674.92</v>
+        <v>145080</v>
       </c>
       <c r="G6" s="5">
         <f>ROUND(E6*F6,2)</f>
         <v/>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1">
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Makine ve ekipman alımı</t>
@@ -4249,14 +4230,14 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>Tünel havalandırma fanı — 4 adet, 138 x 138 x 42 cm, 40.000 m³/h, 1,5 kW, galvanizli çelik kanat, ahtapot sistemli otomatik panjur</t>
+          <t>Havalandırma fanları — Kümes başına 4 adet tünel fanı, 138 x 138 x 42 cm, 40.000 m³/h, 1,5 kW, galvanizli çelik kanat, ahtapot sistemli otomatik panjur</t>
         </is>
       </c>
       <c r="E7" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>76982.48</v>
+        <v>76980</v>
       </c>
       <c r="G7" s="5">
         <f>ROUND(E7*F7,2)</f>
@@ -4274,26 +4255,26 @@
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>HZC-WTR-005</t>
+          <t>HZC-WNT-024</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>Sulama sistemi — 4 hat, hat başına 312 m, 22 x 22 mm hat çapı, 1.560 metal 360° nipel suluk, 4 regülatör, 0,75 kW çift redüktörlü frenli otomatik kaldırma</t>
+          <t>Soğutma petek sistemi (açma-kapama ve petek panelleri dâhil) — Tüplü, dahili devridaimli; 15 cm kalınlık, 150 cm yükseklik, kümes başına 2 x 15 m (45 m² ped alanı), PVC çerçeve, XPS petek kapakları, 2 aktüatör, 2 adet 0,50 kW su pompası</t>
         </is>
       </c>
       <c r="E8" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>145353.3</v>
+        <v>269280</v>
       </c>
       <c r="G8" s="5">
         <f>ROUND(E8*F8,2)</f>
         <v/>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="20" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Makine ve ekipman alımı</t>
@@ -4304,26 +4285,26 @@
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>HZC-WNT-024</t>
+          <t>HZC-WNT-001</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>Soğutma pedi sistemi — Tüplü, dahili devridaimli; 15 cm kalınlık, 150 cm yükseklik, 2 x 15 m uzunluk (45 m² ped alanı), PVC çerçeve, XPS petek kapakları, 2 aktüatör, 2 adet 0,50 kW su pompası</t>
+          <t>Hava klape sistemi (açma-kapama hattı dâhil) — Kümes başına 30 adet 26 x 56 cm izolasyonlu plastik klape, 2 aktüatörlü açma-kapama, 161 m hat</t>
         </is>
       </c>
       <c r="E9" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>269272.63</v>
+        <v>40581.3</v>
       </c>
       <c r="G9" s="5">
         <f>ROUND(E9*F9,2)</f>
         <v/>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="20" customHeight="1">
       <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Makine ve ekipman alımı</t>
@@ -4334,19 +4315,19 @@
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>HZC-WNT-001</t>
+          <t>HZC-SLO-004</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>Klape sistemi — 30 adet 26 x 56 cm izolasyonlu plastik klape, klape başına 1.750 m³/h (30 x 1.750 = 52.500 m³/h, mekanik projedeki 46.717 m³/h ihtiyacının üzerinde), 2 aktüatörlü açma-kapama, 161 m hat</t>
+          <t>17,67 ton silo ve aktarma grubu — Kümes başına 1 adet galvaniz kaplama sac silo, helezonlu merdiven, 0,75 kW yem nakil motoru, 22 m PVC nakil hattı</t>
         </is>
       </c>
       <c r="E10" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>40581.31</v>
+        <v>172995</v>
       </c>
       <c r="G10" s="5">
         <f>ROUND(E10*F10,2)</f>
@@ -4364,68 +4345,128 @@
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>HZC-SLO-004</t>
+          <t>HZC-LGHT-01</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>Yem silosu ve nakil sistemi — En az 17,77 ton galvaniz kaplama sac silo, helezonlu merdiven, 0,75 kW yem nakil motoru, 22 m PVC nakil hattı</t>
+          <t>Aydınlatma sistemi — Kümes başına 56 adet E27 / LED lamba (7-12 W), contalı duy, 266 m kablo</t>
         </is>
       </c>
       <c r="E11" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>172996.93</v>
+        <v>29260</v>
       </c>
       <c r="G11" s="5">
         <f>ROUND(E11*F11,2)</f>
         <v/>
       </c>
     </row>
-    <row r="12" ht="14" customHeight="1">
+    <row r="12" ht="30" customHeight="1">
       <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Makine ve ekipman alımı</t>
         </is>
       </c>
       <c r="B12" s="19" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>HZC-HEA-004</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>Montaj ve nakliye — Kümes montajı ve nakliye bedelleri</t>
+          <t>Isıtma sistemi — 350.000 kcal/h — Kümes başına 1 adet; en az 1.700 m² ısıtma alanı, 350.000 kcal/h, 5,5 kW fan motoru, 21.000 m³/h basma, üç geçişli kazan, 10 mm cehennemlik</t>
         </is>
       </c>
       <c r="E12" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>225000</v>
+        <v>472210</v>
       </c>
       <c r="G12" s="5">
         <f>ROUND(E12*F12,2)</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="21" t="n"/>
-      <c r="B13" s="21" t="n"/>
-      <c r="C13" s="22" t="inlineStr">
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Makine ve ekipman alımı</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>HZC-COM-004</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Kümes otomasyonu ve bilgisayar sistemi — HZC-70 işlemcili; 5 sıcaklık, 1 nem, 1 basınç ve 1 CO2 sensörü, alarm sistemi, uzaktan erişim, PLC kontrol, raporlama ve analiz</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>263300</v>
+      </c>
+      <c r="G13" s="5">
+        <f>ROUND(E13*F13,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="14" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Makine ve ekipman alımı</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>İşçilik ve nakliye — Kümes montajı ve nakliye bedelleri</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>225000</v>
+      </c>
+      <c r="G14" s="5">
+        <f>ROUND(E14*F14,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="n"/>
+      <c r="B15" s="21" t="n"/>
+      <c r="C15" s="22" t="inlineStr">
         <is>
           <t>MAKİNE-EKİPMAN TOPLAMI (KDV hariç)</t>
         </is>
       </c>
-      <c r="D13" s="21" t="n"/>
-      <c r="E13" s="21" t="n"/>
-      <c r="F13" s="21" t="n"/>
-      <c r="G13" s="9">
-        <f>SUM(G5:G12)</f>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="21" t="n"/>
+      <c r="G15" s="9">
+        <f>SUM(G5:G14)</f>
         <v/>
       </c>
     </row>
@@ -7000,7 +7041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="66" customWidth="1" min="1" max="1"/>
@@ -7053,7 +7094,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>25183092.46</v>
+        <v>25480113.85</v>
       </c>
       <c r="C5" s="6">
         <f>B5/52.7585</f>
@@ -7110,7 +7151,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>2885847.21</v>
+        <v>3892868.6</v>
       </c>
       <c r="C8" s="6">
         <f>B8/52.7585</f>
@@ -7123,76 +7164,57 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>Hibe dışı kümes ısıtma sistemi — ayrı lot</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>710000</v>
-      </c>
-      <c r="C9" s="6">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>UYGUN OLMAYAN HARCAMA — toplam</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>9759921.35</v>
+      </c>
+      <c r="C9" s="10">
         <f>B9/52.7585</f>
         <v/>
       </c>
-      <c r="D9" s="17" t="inlineStr">
-        <is>
-          <t>Proforma fatura</t>
+      <c r="D9" s="25" t="inlineStr">
+        <is>
+          <t>Öz kaynak</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
-        <is>
-          <t>UYGUN OLMAYAN HARCAMA — toplam</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="n">
-        <v>9462899.960000001</v>
-      </c>
-      <c r="C10" s="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>IPARD III broyler uygun harcama üst limiti (375.000,00 Avro) — uygun harcama limitin altındadır</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>19784437.5</v>
+      </c>
+      <c r="C10" s="6">
         <f>B10/52.7585</f>
         <v/>
       </c>
-      <c r="D10" s="25" t="inlineStr">
-        <is>
-          <t>Öz kaynak</t>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>Çağrı rehberi</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>IPARD III broyler uygun harcama üst limiti (375.000,00 Avro) — uygun harcama limitin altındadır</t>
+          <t>KDV — IPARD'da uygun harcama değildir</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>19784437.5</v>
+        <v>5096022.77</v>
       </c>
       <c r="C11" s="6">
         <f>B11/52.7585</f>
         <v/>
       </c>
       <c r="D11" s="17" t="inlineStr">
-        <is>
-          <t>Çağrı rehberi</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>KDV — IPARD'da uygun harcama değildir</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>5036618.49</v>
-      </c>
-      <c r="C12" s="6">
-        <f>B12/52.7585</f>
-        <v/>
-      </c>
-      <c r="D12" s="17" t="inlineStr">
         <is>
           <t>Öz kaynak</t>
         </is>

</xml_diff>

<commit_message>
Yayın: makine-ekipman gideri 3.784.288,46 TL
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
+++ b/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>'A3.4-EK Makine-Ekipman'!G15</f>
+        <f>'A3.4-EK Makine-Ekipman'!G14</f>
         <v/>
       </c>
       <c r="C13" s="6">
@@ -4090,7 +4090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4177,7 +4177,7 @@
         <v>2</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>251748</v>
+        <v>250062.03</v>
       </c>
       <c r="G5" s="5">
         <f>ROUND(E5*F5,2)</f>
@@ -4207,7 +4207,7 @@
         <v>2</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>145080</v>
+        <v>145353.3</v>
       </c>
       <c r="G6" s="5">
         <f>ROUND(E6*F6,2)</f>
@@ -4237,7 +4237,7 @@
         <v>2</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>76980</v>
+        <v>76982.48</v>
       </c>
       <c r="G7" s="5">
         <f>ROUND(E7*F7,2)</f>
@@ -4260,14 +4260,14 @@
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>Soğutma petek sistemi (açma-kapama ve petek panelleri dâhil) — Tüplü, dahili devridaimli; 15 cm kalınlık, 150 cm yükseklik, kümes başına 2 x 15 m (45 m² ped alanı), PVC çerçeve, XPS petek kapakları, 2 aktüatör, 2 adet 0,50 kW su pompası</t>
+          <t>Soğutma petekleri ve kapatma sistemi — Tüplü, dahili devridaimli; 15 cm kalınlık, 150 cm yükseklik, kümes başına 2 x 15 m (45 m² ped alanı), PVC çerçeve, XPS petek kapakları, 2 aktüatör, 2 adet 0,50 kW su pompası</t>
         </is>
       </c>
       <c r="E8" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>269280</v>
+        <v>269272.63</v>
       </c>
       <c r="G8" s="5">
         <f>ROUND(E8*F8,2)</f>
@@ -4320,21 +4320,21 @@
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>17,67 ton silo ve aktarma grubu — Kümes başına 1 adet galvaniz kaplama sac silo, helezonlu merdiven, 0,75 kW yem nakil motoru, 22 m PVC nakil hattı</t>
+          <t>Silo ve aktarma sistemi — 17,67 ton — Kümes başına 1 adet galvaniz kaplama sac silo, helezonlu merdiven, 0,75 kW yem nakil motoru, 22 m PVC nakil hattı</t>
         </is>
       </c>
       <c r="E10" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>172995</v>
+        <v>172996.93</v>
       </c>
       <c r="G10" s="5">
         <f>ROUND(E10*F10,2)</f>
         <v/>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
+    <row r="11" ht="30" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Makine ve ekipman alımı</t>
@@ -4345,19 +4345,19 @@
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>HZC-LGHT-01</t>
+          <t>HZC-HEA-004</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>Aydınlatma sistemi — Kümes başına 56 adet E27 / LED lamba (7-12 W), contalı duy, 266 m kablo</t>
+          <t>Isıtma sistemi — 350.000 kcal/h — Kümes başına 1 adet katı yakıtlı ısıtma kazanı, brandalı model, 171 m hava kanalı; en az 1.700 m² ısıtma alanı, 5,5 kW fan motoru, 21.000 m³/h basma, üç geçişli kazan</t>
         </is>
       </c>
       <c r="E11" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>29260</v>
+        <v>472211.18</v>
       </c>
       <c r="G11" s="5">
         <f>ROUND(E11*F11,2)</f>
@@ -4375,26 +4375,26 @@
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>HZC-HEA-004</t>
+          <t>HZC-COM-004</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>Isıtma sistemi — 350.000 kcal/h — Kümes başına 1 adet; en az 1.700 m² ısıtma alanı, 350.000 kcal/h, 5,5 kW fan motoru, 21.000 m³/h basma, üç geçişli kazan, 10 mm cehennemlik</t>
+          <t>Kümes otomasyonu ve bilgisayar sistemi — HZC-70 işlemcili pano; 5 ısı, 1 nem, 1 basınç sensörü, ek alarm sensörü, sensör kablolamaları, uzaktan erişim, PLC kontrol, raporlama ve analiz</t>
         </is>
       </c>
       <c r="E12" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>472210</v>
+        <v>239684.38</v>
       </c>
       <c r="G12" s="5">
         <f>ROUND(E12*F12,2)</f>
         <v/>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
+    <row r="13" ht="14" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Makine ve ekipman alımı</t>
@@ -4405,68 +4405,38 @@
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>HZC-COM-004</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>Kümes otomasyonu ve bilgisayar sistemi — HZC-70 işlemcili; 5 sıcaklık, 1 nem, 1 basınç ve 1 CO2 sensörü, alarm sistemi, uzaktan erişim, PLC kontrol, raporlama ve analiz</t>
+          <t>İşçilik ve nakliye — Kümes montajı ve nakliye bedelleri</t>
         </is>
       </c>
       <c r="E13" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>263300</v>
+        <v>225000</v>
       </c>
       <c r="G13" s="5">
         <f>ROUND(E13*F13,2)</f>
         <v/>
       </c>
     </row>
-    <row r="14" ht="14" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
-        <is>
-          <t>Makine ve ekipman alımı</t>
-        </is>
-      </c>
-      <c r="B14" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="C14" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D14" s="16" t="inlineStr">
-        <is>
-          <t>İşçilik ve nakliye — Kümes montajı ve nakliye bedelleri</t>
-        </is>
-      </c>
-      <c r="E14" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>225000</v>
-      </c>
-      <c r="G14" s="5">
-        <f>ROUND(E14*F14,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="n"/>
-      <c r="B15" s="21" t="n"/>
-      <c r="C15" s="22" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="21" t="n"/>
+      <c r="B14" s="21" t="n"/>
+      <c r="C14" s="22" t="inlineStr">
         <is>
           <t>MAKİNE-EKİPMAN TOPLAMI (KDV hariç)</t>
         </is>
       </c>
-      <c r="D15" s="21" t="n"/>
-      <c r="E15" s="21" t="n"/>
-      <c r="F15" s="21" t="n"/>
-      <c r="G15" s="9">
-        <f>SUM(G5:G14)</f>
+      <c r="D14" s="21" t="n"/>
+      <c r="E14" s="21" t="n"/>
+      <c r="F14" s="21" t="n"/>
+      <c r="G14" s="9">
+        <f>SUM(G5:G13)</f>
         <v/>
       </c>
     </row>
@@ -7094,7 +7064,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>25480113.85</v>
+        <v>25371533.71</v>
       </c>
       <c r="C5" s="6">
         <f>B5/52.7585</f>
@@ -7151,7 +7121,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>3892868.6</v>
+        <v>3784288.46</v>
       </c>
       <c r="C8" s="6">
         <f>B8/52.7585</f>
@@ -7170,7 +7140,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>9759921.35</v>
+        <v>9651341.210000001</v>
       </c>
       <c r="C9" s="10">
         <f>B9/52.7585</f>
@@ -7208,7 +7178,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>5096022.77</v>
+        <v>5074306.74</v>
       </c>
       <c r="C11" s="6">
         <f>B11/52.7585</f>

</xml_diff>

<commit_message>
Yayın: beyan belgeleri TKDK başvuru ekranlarına eşitlendi (EKRAN-UYUMU)
Hibe dışı yapım işleri 5.867.052,75 -> 5.541.091,09 TL (ÖP-15 foseptik
tankı ve dokuz satırlık sıhhi tesisat beyan belgelerinden çıkarıldı),
makine-ekipman 3.784.288,46 -> 3.784.288,48 TL (ekrandaki miktar
bölünmesi işlendi). Uygun harcama değişmedi: 297.965 Avro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
+++ b/belgeler/21_A3_UYGUN_HARCAMALAR.xlsx
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>'A3.4-EK Yapım'!H64</f>
+        <f>'A3.4-EK Yapım'!H53</f>
         <v/>
       </c>
       <c r="C12" s="6">
@@ -4207,7 +4207,7 @@
         <v>2</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>145353.3</v>
+        <v>145353.32</v>
       </c>
       <c r="G6" s="5">
         <f>ROUND(E6*F6,2)</f>
@@ -4267,7 +4267,7 @@
         <v>2</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>269272.63</v>
+        <v>269272.64</v>
       </c>
       <c r="G8" s="5">
         <f>ROUND(E8*F8,2)</f>
@@ -4327,7 +4327,7 @@
         <v>2</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>172996.93</v>
+        <v>172996.92</v>
       </c>
       <c r="G10" s="5">
         <f>ROUND(E10*F10,2)</f>
@@ -4387,7 +4387,7 @@
         <v>2</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>239684.38</v>
+        <v>239684.37</v>
       </c>
       <c r="G12" s="5">
         <f>ROUND(E12*F12,2)</f>
@@ -4454,7 +4454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4477,7 +4477,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Kümes A ve B blokları dışındaki yapılar ile bu iki bloktan hibe kapsamı dışına çıkarılan pozlar. Bu imalatlar yapılmaya devam eder; teklif alma usulüne tabi değildir, proforma fatura ile beyan edilir ve tamamı öz kaynaktan karşılanır. Birim fiyatlar, hibe kapsamındaki işlerle aynı esasa göre kurulmuştur: ÇŞB 2026 ve TKDK 17.02.2026 kitap fiyatlarına %16 tenzilat uygulanmıştır. Sayfanın sonundaki SIHHİ TESİSAT bölümü keşif özetinde yer almaz: miktarları onaylı sıhhi tesisat projesinden, birim fiyatları piyasa araştırmasından gelir; kitap fiyatı olmadığı için o kalemlere tenzilat uygulanmaz. Bu sayfa 36 numaralı proforma ile kuruşu kuruşuna aynıdır.</t>
+          <t>Kümes A ve B blokları dışındaki yapılar ile bu iki bloktan hibe kapsamı dışına çıkarılan pozlar. Bu imalatlar yapılmaya devam eder; teklif alma usulüne tabi değildir, proforma fatura ile beyan edilir ve tamamı öz kaynaktan karşılanır. Birim fiyatlar, hibe kapsamındaki işlerle aynı esasa göre kurulmuştur: ÇŞB 2026 ve TKDK 17.02.2026 kitap fiyatlarına %16 tenzilat uygulanmıştır. Bu sayfa 36 numaralı proforma ile ve TKDK Online Başvuru Sistemine girilen uygun olmayan yapım işleri listesiyle kuruşu kuruşuna aynıdır.</t>
         </is>
       </c>
     </row>
@@ -5893,25 +5893,25 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="30" customHeight="1">
+    <row r="42" ht="20" customHeight="1">
       <c r="A42" s="16" t="inlineStr">
         <is>
-          <t>Kanalizasyon işleri</t>
+          <t>Elektrik tesisatı ve aydınlatma</t>
         </is>
       </c>
       <c r="B42" s="17" t="inlineStr">
         <is>
-          <t>Foseptik</t>
+          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
         </is>
       </c>
       <c r="C42" s="18" t="inlineStr">
         <is>
-          <t>ÖP-15</t>
+          <t>35.100.1104</t>
         </is>
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>Prefabrik polietilen sızdırmaz foseptik tankı — 6 m³, rotasyon kalıplı, temini, yerine konulması ve giriş-çıkış bağlantılarının yapılması</t>
+          <t>Ana dağıtım panosu (dikili tip galvanizli sac, en az 700 mm en, 400 mm derinlik) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="E42" s="19" t="inlineStr">
@@ -5923,7 +5923,7 @@
         <v>1</v>
       </c>
       <c r="G42" s="5" t="n">
-        <v>76961.66</v>
+        <v>31602.33</v>
       </c>
       <c r="H42" s="5">
         <f>ROUND(F42*G42,2)</f>
@@ -5943,12 +5943,12 @@
       </c>
       <c r="C43" s="18" t="inlineStr">
         <is>
-          <t>35.100.1104</t>
+          <t>35.100.2106</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>Ana dağıtım panosu (dikili tip galvanizli sac, en az 700 mm en, 400 mm derinlik) (%25 müteahhit kârı dahil)</t>
+          <t>Sayaç panosu (sıva üstü galvanizli sac tablo, 0,50-0,60 m²) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="E43" s="19" t="inlineStr">
@@ -5960,7 +5960,7 @@
         <v>1</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>31602.33</v>
+        <v>8179.25</v>
       </c>
       <c r="H43" s="5">
         <f>ROUND(F43*G43,2)</f>
@@ -5980,12 +5980,12 @@
       </c>
       <c r="C44" s="18" t="inlineStr">
         <is>
-          <t>35.100.2106</t>
+          <t>35.135.3201</t>
         </is>
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
-          <t>Sayaç panosu (sıva üstü galvanizli sac tablo, 0,50-0,60 m²) (%25 müteahhit kârı dahil)</t>
+          <t>Üç fazlı zaman tarifeli elektronik aktif sayaç, en az 5(100) A, 3x230/400 V (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="E44" s="19" t="inlineStr">
@@ -5997,7 +5997,7 @@
         <v>1</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>8179.25</v>
+        <v>1504.15</v>
       </c>
       <c r="H44" s="5">
         <f>ROUND(F44*G44,2)</f>
@@ -6017,12 +6017,12 @@
       </c>
       <c r="C45" s="18" t="inlineStr">
         <is>
-          <t>35.135.3201</t>
+          <t>35.110.1104</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>Üç fazlı zaman tarifeli elektronik aktif sayaç, en az 5(100) A, 3x230/400 V (%25 müteahhit kârı dahil)</t>
+          <t>Termik-manyetik kompakt şalter 3x160 A, Icu 35 kA — ana giriş (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="E45" s="19" t="inlineStr">
@@ -6034,7 +6034,7 @@
         <v>1</v>
       </c>
       <c r="G45" s="5" t="n">
-        <v>1504.15</v>
+        <v>4753.16</v>
       </c>
       <c r="H45" s="5">
         <f>ROUND(F45*G45,2)</f>
@@ -6054,12 +6054,12 @@
       </c>
       <c r="C46" s="18" t="inlineStr">
         <is>
-          <t>35.110.1104</t>
+          <t>35.115.1003</t>
         </is>
       </c>
       <c r="D46" s="16" t="inlineStr">
         <is>
-          <t>Termik-manyetik kompakt şalter 3x160 A, Icu 35 kA — ana giriş (%25 müteahhit kârı dahil)</t>
+          <t>Kaçak akım koruma şalteri 2x63 A, 30 mA (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="E46" s="19" t="inlineStr">
@@ -6068,10 +6068,10 @@
         </is>
       </c>
       <c r="F46" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>4753.16</v>
+        <v>1079.2</v>
       </c>
       <c r="H46" s="5">
         <f>ROUND(F46*G46,2)</f>
@@ -6091,24 +6091,24 @@
       </c>
       <c r="C47" s="18" t="inlineStr">
         <is>
-          <t>35.115.1003</t>
+          <t>35.140.3105</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>Kaçak akım koruma şalteri 2x63 A, 30 mA (%25 müteahhit kârı dahil)</t>
+          <t>YVV (NYY) 1 kV yeraltı kablosu ile besleme hattı tesisi — 1x35 mm² (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="E47" s="19" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="F47" s="20" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>1079.2</v>
+        <v>277.15</v>
       </c>
       <c r="H47" s="5">
         <f>ROUND(F47*G47,2)</f>
@@ -6128,12 +6128,12 @@
       </c>
       <c r="C48" s="18" t="inlineStr">
         <is>
-          <t>35.140.3105</t>
+          <t>35.140.3101</t>
         </is>
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>YVV (NYY) 1 kV yeraltı kablosu ile besleme hattı tesisi — 1x35 mm² (%25 müteahhit kârı dahil)</t>
+          <t>YVV (NYY) 1 kV yeraltı kablosu ile besleme hattı tesisi — 1x6 mm² (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="E48" s="19" t="inlineStr">
@@ -6145,7 +6145,7 @@
         <v>50</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>277.15</v>
+        <v>51.25</v>
       </c>
       <c r="H48" s="5">
         <f>ROUND(F48*G48,2)</f>
@@ -6165,24 +6165,24 @@
       </c>
       <c r="C49" s="18" t="inlineStr">
         <is>
-          <t>35.140.3101</t>
+          <t>35.172.1706</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
-          <t>YVV (NYY) 1 kV yeraltı kablosu ile besleme hattı tesisi — 1x6 mm² (%25 müteahhit kârı dahil)</t>
+          <t>Aydınlatma direği — taban çapı en az 80 mm, yükseklik en az 4,00 m (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="E49" s="19" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="F49" s="20" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="G49" s="5" t="n">
-        <v>51.25</v>
+        <v>6229.12</v>
       </c>
       <c r="H49" s="5">
         <f>ROUND(F49*G49,2)</f>
@@ -6202,12 +6202,12 @@
       </c>
       <c r="C50" s="18" t="inlineStr">
         <is>
-          <t>35.172.1706</t>
+          <t>35.170.4002</t>
         </is>
       </c>
       <c r="D50" s="16" t="inlineStr">
         <is>
-          <t>Aydınlatma direği — taban çapı en az 80 mm, yükseklik en az 4,00 m (%25 müteahhit kârı dahil)</t>
+          <t>LED projektör, ışık akısı en az 5100 lm (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="E50" s="19" t="inlineStr">
@@ -6219,7 +6219,7 @@
         <v>4</v>
       </c>
       <c r="G50" s="5" t="n">
-        <v>6229.12</v>
+        <v>7632.76</v>
       </c>
       <c r="H50" s="5">
         <f>ROUND(F50*G50,2)</f>
@@ -6234,17 +6234,17 @@
       </c>
       <c r="B51" s="17" t="inlineStr">
         <is>
-          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
+          <t>Kümes A Blok</t>
         </is>
       </c>
       <c r="C51" s="18" t="inlineStr">
         <is>
-          <t>35.170.4002</t>
+          <t>35.120.2016</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>LED projektör, ışık akısı en az 5100 lm (%25 müteahhit kârı dahil)</t>
+          <t>Otomatik transfer şalteri 4 x 200 A (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="E51" s="19" t="inlineStr">
@@ -6253,10 +6253,10 @@
         </is>
       </c>
       <c r="F51" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G51" s="5" t="n">
-        <v>7632.76</v>
+        <v>38544.21</v>
       </c>
       <c r="H51" s="5">
         <f>ROUND(F51*G51,2)</f>
@@ -6271,7 +6271,7 @@
       </c>
       <c r="B52" s="17" t="inlineStr">
         <is>
-          <t>Kümes A Blok</t>
+          <t>Kümes B Blok</t>
         </is>
       </c>
       <c r="C52" s="18" t="inlineStr">
@@ -6300,403 +6300,25 @@
         <v/>
       </c>
     </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="16" t="inlineStr">
-        <is>
-          <t>Elektrik tesisatı ve aydınlatma</t>
-        </is>
-      </c>
-      <c r="B53" s="17" t="inlineStr">
-        <is>
-          <t>Kümes B Blok</t>
-        </is>
-      </c>
-      <c r="C53" s="18" t="inlineStr">
-        <is>
-          <t>35.120.2016</t>
-        </is>
-      </c>
-      <c r="D53" s="16" t="inlineStr">
-        <is>
-          <t>Otomatik transfer şalteri 4 x 200 A (%25 müteahhit kârı dahil)</t>
-        </is>
-      </c>
-      <c r="E53" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="F53" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G53" s="5" t="n">
-        <v>38544.21</v>
-      </c>
-      <c r="H53" s="5">
-        <f>ROUND(F53*G53,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="1" t="inlineStr">
-        <is>
-          <t>SIHHİ TESİSAT — keşif özetinde yer almaz; miktarlar onaylı sıhhi tesisat projesinden, birim fiyatlar piyasa araştırmasından (kitap fiyatı olmadığı için %16 tenzilat uygulanmaz)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="17" t="inlineStr">
-        <is>
-          <t>Sıhhi tesisat</t>
-        </is>
-      </c>
-      <c r="B55" s="17" t="inlineStr">
-        <is>
-          <t>Kümes A Blok</t>
-        </is>
-      </c>
-      <c r="C55" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D55" s="16" t="inlineStr">
-        <is>
-          <t>Temiz su tesisatı — PPRC boru ve ek parçaları, 1/2" - 1 1/4" kolon ve kat tesisatı, küresel vanalar, boru askı ve kılıfları (kolon şemasına göre)</t>
-        </is>
-      </c>
-      <c r="E55" s="19" t="inlineStr">
-        <is>
-          <t>tk</t>
-        </is>
-      </c>
-      <c r="F55" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G55" s="5" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H55" s="5">
-        <f>ROUND(F55*G55,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="17" t="inlineStr">
-        <is>
-          <t>Sıhhi tesisat</t>
-        </is>
-      </c>
-      <c r="B56" s="17" t="inlineStr">
-        <is>
-          <t>Kümes A Blok</t>
-        </is>
-      </c>
-      <c r="C56" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D56" s="16" t="inlineStr">
-        <is>
-          <t>Pis su tesisatı — Ø50 / Ø70 / Ø100 sert PVC boru, kolon ve yatay hatlar, temizleme kapakları, yer süzgeçleri</t>
-        </is>
-      </c>
-      <c r="E56" s="19" t="inlineStr">
-        <is>
-          <t>tk</t>
-        </is>
-      </c>
-      <c r="F56" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G56" s="5" t="n">
-        <v>27000</v>
-      </c>
-      <c r="H56" s="5">
-        <f>ROUND(F56*G56,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="17" t="inlineStr">
-        <is>
-          <t>Sıhhi tesisat</t>
-        </is>
-      </c>
-      <c r="B57" s="17" t="inlineStr">
-        <is>
-          <t>Kümes A Blok</t>
-        </is>
-      </c>
-      <c r="C57" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D57" s="16" t="inlineStr">
-        <is>
-          <t>Termosifon — sıcak su üretimi (proje raporu: sıcak su hatları termosifon vasıtasıyla)</t>
-        </is>
-      </c>
-      <c r="E57" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="F57" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G57" s="5" t="n">
-        <v>13000</v>
-      </c>
-      <c r="H57" s="5">
-        <f>ROUND(F57*G57,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58" ht="30" customHeight="1">
-      <c r="A58" s="17" t="inlineStr">
-        <is>
-          <t>Sıhhi tesisat</t>
-        </is>
-      </c>
-      <c r="B58" s="17" t="inlineStr">
-        <is>
-          <t>Kümes B Blok</t>
-        </is>
-      </c>
-      <c r="C58" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D58" s="16" t="inlineStr">
-        <is>
-          <t>Temiz su tesisatı — PPRC boru ve ek parçaları, 1/2" - 1 1/4" kolon ve kat tesisatı, küresel vanalar, boru askı ve kılıfları (kolon şemasına göre)</t>
-        </is>
-      </c>
-      <c r="E58" s="19" t="inlineStr">
-        <is>
-          <t>tk</t>
-        </is>
-      </c>
-      <c r="F58" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G58" s="5" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H58" s="5">
-        <f>ROUND(F58*G58,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="A59" s="17" t="inlineStr">
-        <is>
-          <t>Sıhhi tesisat</t>
-        </is>
-      </c>
-      <c r="B59" s="17" t="inlineStr">
-        <is>
-          <t>Kümes B Blok</t>
-        </is>
-      </c>
-      <c r="C59" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D59" s="16" t="inlineStr">
-        <is>
-          <t>Pis su tesisatı — Ø50 / Ø70 / Ø100 sert PVC boru, kolon ve yatay hatlar, temizleme kapakları, yer süzgeçleri</t>
-        </is>
-      </c>
-      <c r="E59" s="19" t="inlineStr">
-        <is>
-          <t>tk</t>
-        </is>
-      </c>
-      <c r="F59" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G59" s="5" t="n">
-        <v>27000</v>
-      </c>
-      <c r="H59" s="5">
-        <f>ROUND(F59*G59,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" ht="20" customHeight="1">
-      <c r="A60" s="17" t="inlineStr">
-        <is>
-          <t>Sıhhi tesisat</t>
-        </is>
-      </c>
-      <c r="B60" s="17" t="inlineStr">
-        <is>
-          <t>Kümes B Blok</t>
-        </is>
-      </c>
-      <c r="C60" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D60" s="16" t="inlineStr">
-        <is>
-          <t>Termosifon — sıcak su üretimi (proje raporu: sıcak su hatları termosifon vasıtasıyla)</t>
-        </is>
-      </c>
-      <c r="E60" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="F60" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G60" s="5" t="n">
-        <v>13000</v>
-      </c>
-      <c r="H60" s="5">
-        <f>ROUND(F60*G60,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" ht="14" customHeight="1">
-      <c r="A61" s="17" t="inlineStr">
-        <is>
-          <t>Sıhhi tesisat</t>
-        </is>
-      </c>
-      <c r="B61" s="17" t="inlineStr">
-        <is>
-          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
-        </is>
-      </c>
-      <c r="C61" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D61" s="16" t="inlineStr">
-        <is>
-          <t>Şebeke su bağlantısı ve 2" su sayacı — temiz su girişi 80 YB</t>
-        </is>
-      </c>
-      <c r="E61" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="F61" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G61" s="5" t="n">
-        <v>26000</v>
-      </c>
-      <c r="H61" s="5">
-        <f>ROUND(F61*G61,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" ht="14" customHeight="1">
-      <c r="A62" s="17" t="inlineStr">
-        <is>
-          <t>Sıhhi tesisat</t>
-        </is>
-      </c>
-      <c r="B62" s="17" t="inlineStr">
-        <is>
-          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
-        </is>
-      </c>
-      <c r="C62" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D62" s="16" t="inlineStr">
-        <is>
-          <t>Hidrofor — Q = 2 m³/h, P = 33-38 mSS</t>
-        </is>
-      </c>
-      <c r="E62" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="F62" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G62" s="5" t="n">
-        <v>48000</v>
-      </c>
-      <c r="H62" s="5">
-        <f>ROUND(F62*G62,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" ht="14" customHeight="1">
-      <c r="A63" s="17" t="inlineStr">
-        <is>
-          <t>Sıhhi tesisat</t>
-        </is>
-      </c>
-      <c r="B63" s="17" t="inlineStr">
-        <is>
-          <t>Çevre Düzenlemesi ve Saha Altyapısı</t>
-        </is>
-      </c>
-      <c r="C63" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D63" s="16" t="inlineStr">
-        <is>
-          <t>Tesisat hidroforu — 0,3 m³/h, 30 mSS (3A)</t>
-        </is>
-      </c>
-      <c r="E63" s="19" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="F63" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G63" s="5" t="n">
-        <v>19000</v>
-      </c>
-      <c r="H63" s="5">
-        <f>ROUND(F63*G63,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="21" t="n"/>
-      <c r="B64" s="21" t="n"/>
-      <c r="C64" s="21" t="n"/>
-      <c r="D64" s="22" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="21" t="n"/>
+      <c r="B53" s="21" t="n"/>
+      <c r="C53" s="21" t="n"/>
+      <c r="D53" s="22" t="inlineStr">
         <is>
           <t>HİBE DIŞI YAPIM İŞLERİ TOPLAMI (KDV hariç)</t>
         </is>
       </c>
-      <c r="E64" s="21" t="n"/>
-      <c r="F64" s="21" t="n"/>
-      <c r="G64" s="21" t="n"/>
-      <c r="H64" s="9">
-        <f>SUM(H5:H63)</f>
+      <c r="E53" s="21" t="n"/>
+      <c r="F53" s="21" t="n"/>
+      <c r="G53" s="21" t="n"/>
+      <c r="H53" s="9">
+        <f>SUM(H5:H52)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A54:H54"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7064,7 +6686,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>25371533.71</v>
+        <v>25045572.07</v>
       </c>
       <c r="C5" s="6">
         <f>B5/52.7585</f>
@@ -7102,7 +6724,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>5867052.75</v>
+        <v>5541091.09</v>
       </c>
       <c r="C7" s="6">
         <f>B7/52.7585</f>
@@ -7121,7 +6743,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>3784288.46</v>
+        <v>3784288.48</v>
       </c>
       <c r="C8" s="6">
         <f>B8/52.7585</f>
@@ -7140,7 +6762,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>9651341.210000001</v>
+        <v>9325379.57</v>
       </c>
       <c r="C9" s="10">
         <f>B9/52.7585</f>
@@ -7178,7 +6800,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>5074306.74</v>
+        <v>5009114.41</v>
       </c>
       <c r="C11" s="6">
         <f>B11/52.7585</f>

</xml_diff>